<commit_message>
Complete burn simulation: feed losses, NHNE injector, CEA, chamber balance, nozzle, startup ramp, vapor tail, plots
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="88">
   <si>
     <t xml:space="preserve">SIMULATION SETUP</t>
   </si>
@@ -32,7 +32,7 @@
     <t xml:space="preserve">Sweep Setup</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuel Properties</t>
+    <t xml:space="preserve">Propellant Properties</t>
   </si>
   <si>
     <t xml:space="preserve">Isopropanol</t>
@@ -83,37 +83,55 @@
     <t xml:space="preserve">Ambient Conditions</t>
   </si>
   <si>
+    <t xml:space="preserve">Oxidizer Dynamic Viscosity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N20 @50F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Timestep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">s</t>
+  </si>
+  <si>
     <t xml:space="preserve">Efficiencies and Blowdown Model</t>
   </si>
   <si>
-    <t xml:space="preserve">Timestep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s</t>
+    <t xml:space="preserve">Sim Duration</t>
   </si>
   <si>
     <t xml:space="preserve">C* Efficiency</t>
   </si>
   <si>
-    <t xml:space="preserve">Sim Duration</t>
+    <t xml:space="preserve">Ambient Temperature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
   </si>
   <si>
     <t xml:space="preserve">Nozzle Efficiency</t>
   </si>
   <si>
-    <t xml:space="preserve">Ambient Temperature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C</t>
+    <t xml:space="preserve">Nitrous Temperature</t>
   </si>
   <si>
     <t xml:space="preserve">Decay Constant (liquid)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nitrous Temperature</t>
+    <t xml:space="preserve">Ambient Pressure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">psi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambient at FAR</t>
   </si>
   <si>
     <t xml:space="preserve">Decay Constant (vapor)</t>
@@ -122,66 +140,75 @@
     <t xml:space="preserve">1/s</t>
   </si>
   <si>
-    <t xml:space="preserve">Ambient Pressure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">psi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambient at FAR</t>
-  </si>
-  <si>
     <t xml:space="preserve">Feed System ΔP</t>
   </si>
   <si>
-    <t xml:space="preserve">Oxidizer Feed Cv</t>
-  </si>
-  <si>
     <t xml:space="preserve">GEOMETRIC CHARACTERISTICS</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuel Feed Cv</t>
+    <t xml:space="preserve">Ball Valve Cv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Ball Valve K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Ball Valve K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tank OD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer No. Elbows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tank Wall Thickness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel No. Elbows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tank Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrance K-factor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulkhead Insertion Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elbow K-factor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piston Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Sum K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Static Vent Position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measured from tank aft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Sum K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Static Vent Diameter</t>
   </si>
   <si>
     <t xml:space="preserve">Fuel Piston Loss</t>
   </si>
   <si>
-    <t xml:space="preserve">Tank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tank OD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tank Wall Thickness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tank Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bulkhead Insertion Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Piston Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Static Vent Position</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Measured from tank aft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Static Vent Diameter</t>
-  </si>
-  <si>
     <t xml:space="preserve">Oxidizer Length</t>
   </si>
   <si>
@@ -191,13 +218,13 @@
     <t xml:space="preserve">Feed System</t>
   </si>
   <si>
-    <t xml:space="preserve">Ox Line Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ox Line Diameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ox Line Roughness</t>
+    <t xml:space="preserve">Oxidizer Line Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Line Diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Line Roughness</t>
   </si>
   <si>
     <t xml:space="preserve">Fuel Line Length</t>
@@ -267,11 +294,11 @@
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.0000"/>
-    <numFmt numFmtId="168" formatCode="0.00E+00"/>
-    <numFmt numFmtId="169" formatCode="0E+00"/>
-    <numFmt numFmtId="170" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="0.00"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="169" formatCode="0.00E+00"/>
+    <numFmt numFmtId="170" formatCode="0E+00"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -626,6 +653,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -646,14 +677,22 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -663,18 +702,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1171,12 +1198,20 @@
       <c r="H8" s="14"/>
       <c r="I8" s="15"/>
       <c r="K8" s="16"/>
-      <c r="L8" s="19"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="19"/>
-      <c r="O8" s="19"/>
-      <c r="P8" s="19"/>
-      <c r="Q8" s="19"/>
+      <c r="L8" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="M8" s="29"/>
+      <c r="N8" s="29"/>
+      <c r="O8" s="30" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="P8" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q8" s="29" t="s">
+        <v>21</v>
+      </c>
       <c r="R8" s="20"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1197,54 +1232,50 @@
       </c>
       <c r="I9" s="15"/>
       <c r="K9" s="16"/>
-      <c r="L9" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="M9" s="33"/>
-      <c r="N9" s="33"/>
-      <c r="O9" s="33"/>
-      <c r="P9" s="33"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
       <c r="Q9" s="19"/>
       <c r="R9" s="20"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="11"/>
       <c r="C10" s="29" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" s="30" t="n">
         <v>0.01</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F10" s="29"/>
       <c r="G10" s="29"/>
       <c r="H10" s="29"/>
       <c r="I10" s="15"/>
       <c r="K10" s="16"/>
-      <c r="L10" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="M10" s="30" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="N10" s="29"/>
-      <c r="O10" s="29"/>
-      <c r="P10" s="29"/>
-      <c r="Q10" s="29"/>
+      <c r="L10" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="M10" s="33"/>
+      <c r="N10" s="33"/>
+      <c r="O10" s="33"/>
+      <c r="P10" s="33"/>
+      <c r="Q10" s="19"/>
       <c r="R10" s="20"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="11"/>
       <c r="C11" s="29" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D11" s="30" t="n">
         <v>30</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11" s="29"/>
       <c r="G11" s="29"/>
@@ -1252,10 +1283,10 @@
       <c r="I11" s="15"/>
       <c r="K11" s="16"/>
       <c r="L11" s="29" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M11" s="30" t="n">
-        <v>0.95</v>
+        <v>0.65</v>
       </c>
       <c r="N11" s="29"/>
       <c r="O11" s="29"/>
@@ -1266,29 +1297,29 @@
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="11"/>
       <c r="C12" s="29" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D12" s="30" t="n">
         <v>60</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F12" s="34" t="n">
         <f aca="false">(D12-32)/1.8</f>
         <v>15.5555555555556</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H12" s="29"/>
       <c r="I12" s="15"/>
       <c r="K12" s="16"/>
       <c r="L12" s="29" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M12" s="30" t="n">
-        <v>0.7</v>
+        <v>0.95</v>
       </c>
       <c r="N12" s="29"/>
       <c r="O12" s="29"/>
@@ -1299,34 +1330,32 @@
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="11"/>
       <c r="C13" s="29" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D13" s="29" t="n">
         <f aca="false">D12-10</f>
         <v>50</v>
       </c>
       <c r="E13" s="29" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F13" s="34" t="n">
         <f aca="false">(D13-32)/1.8</f>
         <v>10</v>
       </c>
       <c r="G13" s="29" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H13" s="29"/>
       <c r="I13" s="15"/>
       <c r="K13" s="16"/>
       <c r="L13" s="29" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M13" s="30" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N13" s="29" t="s">
-        <v>32</v>
-      </c>
+        <v>0.7</v>
+      </c>
+      <c r="N13" s="29"/>
       <c r="O13" s="29"/>
       <c r="P13" s="29"/>
       <c r="Q13" s="29"/>
@@ -1355,12 +1384,18 @@
       </c>
       <c r="I14" s="15"/>
       <c r="K14" s="16"/>
-      <c r="L14" s="33"/>
-      <c r="M14" s="33"/>
-      <c r="N14" s="33"/>
-      <c r="O14" s="33"/>
-      <c r="P14" s="33"/>
-      <c r="Q14" s="33"/>
+      <c r="L14" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="M14" s="30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N14" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="O14" s="29"/>
+      <c r="P14" s="29"/>
+      <c r="Q14" s="29"/>
       <c r="R14" s="20"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1373,9 +1408,7 @@
       <c r="H15" s="36"/>
       <c r="I15" s="37"/>
       <c r="K15" s="16"/>
-      <c r="L15" s="32" t="s">
-        <v>37</v>
-      </c>
+      <c r="L15" s="33"/>
       <c r="M15" s="33"/>
       <c r="N15" s="33"/>
       <c r="O15" s="33"/>
@@ -1385,25 +1418,23 @@
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K16" s="16"/>
-      <c r="L16" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="M16" s="30" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="N16" s="29"/>
-      <c r="O16" s="29"/>
-      <c r="P16" s="29"/>
-      <c r="Q16" s="29"/>
+      <c r="L16" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="M16" s="33"/>
+      <c r="N16" s="33"/>
+      <c r="O16" s="33"/>
+      <c r="P16" s="33"/>
+      <c r="Q16" s="33"/>
       <c r="R16" s="20"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K17" s="16"/>
       <c r="L17" s="29" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M17" s="30" t="n">
         <v>1.6</v>
@@ -1425,524 +1456,624 @@
       <c r="I18" s="41"/>
       <c r="K18" s="16"/>
       <c r="L18" s="29" t="s">
-        <v>41</v>
-      </c>
-      <c r="M18" s="30" t="n">
-        <v>15</v>
-      </c>
-      <c r="N18" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="O18" s="29" t="n">
-        <f aca="false">M18*6895</f>
-        <v>103425</v>
-      </c>
-      <c r="P18" s="29" t="s">
-        <v>35</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="M18" s="42" t="n">
+        <f aca="false">891 * D32^4 / M17^2</f>
+        <v>3.31923365592957</v>
+      </c>
+      <c r="N18" s="29"/>
+      <c r="O18" s="29"/>
+      <c r="P18" s="29"/>
       <c r="Q18" s="29"/>
       <c r="R18" s="20"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="42"/>
-      <c r="C19" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="44"/>
-      <c r="E19" s="44"/>
-      <c r="F19" s="44"/>
-      <c r="G19" s="44"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="46"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="44" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="45"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="45"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="47"/>
       <c r="K19" s="16"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="19"/>
-      <c r="O19" s="19"/>
-      <c r="P19" s="19"/>
-      <c r="Q19" s="19"/>
+      <c r="L19" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="M19" s="42" t="n">
+        <f aca="false">891 * D35^4 / M17^2</f>
+        <v>0.892006072998047</v>
+      </c>
+      <c r="N19" s="29"/>
+      <c r="O19" s="29"/>
+      <c r="P19" s="29"/>
+      <c r="Q19" s="29"/>
       <c r="R19" s="20"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="42"/>
+      <c r="B20" s="43"/>
       <c r="C20" s="29" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D20" s="30" t="n">
         <v>4</v>
       </c>
       <c r="E20" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F20" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F20" s="48" t="n">
         <f aca="false">D20*0.0254</f>
         <v>0.1016</v>
       </c>
       <c r="G20" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H20" s="29"/>
-      <c r="I20" s="46"/>
+      <c r="I20" s="47"/>
       <c r="K20" s="16"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
-      <c r="O20" s="19"/>
-      <c r="P20" s="19"/>
-      <c r="Q20" s="19"/>
+      <c r="L20" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="M20" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="29"/>
+      <c r="O20" s="29"/>
+      <c r="P20" s="29"/>
+      <c r="Q20" s="29"/>
       <c r="R20" s="20"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="42"/>
+      <c r="B21" s="43"/>
       <c r="C21" s="29" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D21" s="30" t="n">
         <v>0.125</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F21" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F21" s="48" t="n">
         <f aca="false">D21*0.0254</f>
         <v>0.003175</v>
       </c>
       <c r="G21" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H21" s="29"/>
-      <c r="I21" s="46"/>
+      <c r="I21" s="47"/>
       <c r="K21" s="16"/>
-      <c r="L21" s="19"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="19"/>
-      <c r="O21" s="19"/>
-      <c r="P21" s="19"/>
-      <c r="Q21" s="19"/>
+      <c r="L21" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="M21" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="N21" s="29"/>
+      <c r="O21" s="29"/>
+      <c r="P21" s="29"/>
+      <c r="Q21" s="29"/>
       <c r="R21" s="20"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="42"/>
+      <c r="B22" s="43"/>
       <c r="C22" s="29" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D22" s="30" t="n">
         <v>36</v>
       </c>
       <c r="E22" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F22" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F22" s="48" t="n">
         <f aca="false">D22*0.0254</f>
         <v>0.9144</v>
       </c>
       <c r="G22" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H22" s="29"/>
-      <c r="I22" s="46"/>
+      <c r="I22" s="47"/>
       <c r="K22" s="16"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="19"/>
-      <c r="O22" s="19"/>
-      <c r="P22" s="19"/>
-      <c r="Q22" s="19"/>
+      <c r="L22" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="M22" s="30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N22" s="29"/>
+      <c r="O22" s="29"/>
+      <c r="P22" s="29"/>
+      <c r="Q22" s="29"/>
       <c r="R22" s="20"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="42"/>
+      <c r="B23" s="43"/>
       <c r="C23" s="29" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D23" s="30" t="n">
         <v>1.5</v>
       </c>
       <c r="E23" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F23" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F23" s="48" t="n">
         <f aca="false">D23*0.0254</f>
         <v>0.0381</v>
       </c>
       <c r="G23" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H23" s="29"/>
-      <c r="I23" s="46"/>
+      <c r="I23" s="47"/>
       <c r="K23" s="16"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="19"/>
-      <c r="O23" s="19"/>
-      <c r="P23" s="19"/>
-      <c r="Q23" s="19"/>
+      <c r="L23" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="M23" s="30" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N23" s="29"/>
+      <c r="O23" s="29"/>
+      <c r="P23" s="29"/>
+      <c r="Q23" s="29"/>
       <c r="R23" s="20"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="42"/>
+      <c r="B24" s="43"/>
       <c r="C24" s="29" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D24" s="30" t="n">
         <v>3</v>
       </c>
       <c r="E24" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F24" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F24" s="48" t="n">
         <f aca="false">D24*0.0254</f>
         <v>0.0762</v>
       </c>
       <c r="G24" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H24" s="29"/>
-      <c r="I24" s="46"/>
+      <c r="I24" s="47"/>
       <c r="K24" s="16"/>
-      <c r="L24" s="19"/>
-      <c r="M24" s="19"/>
-      <c r="N24" s="19"/>
-      <c r="O24" s="19"/>
-      <c r="P24" s="19"/>
-      <c r="Q24" s="19"/>
+      <c r="L24" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="M24" s="42" t="n">
+        <f aca="false">M23*M20+M18 + M22</f>
+        <v>3.81923365592957</v>
+      </c>
+      <c r="N24" s="29"/>
+      <c r="O24" s="29"/>
+      <c r="P24" s="29"/>
+      <c r="Q24" s="29"/>
       <c r="R24" s="20"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="42"/>
+      <c r="B25" s="43"/>
       <c r="C25" s="29" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D25" s="30" t="n">
         <v>22.5</v>
       </c>
       <c r="E25" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F25" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F25" s="48" t="n">
         <f aca="false">D25*0.0254</f>
         <v>0.5715</v>
       </c>
       <c r="G25" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H25" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="I25" s="46"/>
+        <v>58</v>
+      </c>
+      <c r="I25" s="47"/>
       <c r="K25" s="16"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="19"/>
-      <c r="N25" s="19"/>
-      <c r="O25" s="19"/>
-      <c r="P25" s="19"/>
-      <c r="Q25" s="19"/>
+      <c r="L25" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="M25" s="42" t="n">
+        <f aca="false">M19 + M23*M21 + M22</f>
+        <v>2.99200607299805</v>
+      </c>
+      <c r="N25" s="29"/>
+      <c r="O25" s="29"/>
+      <c r="P25" s="29"/>
+      <c r="Q25" s="29"/>
       <c r="R25" s="20"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="42"/>
+      <c r="B26" s="43"/>
       <c r="C26" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="D26" s="48" t="n">
+        <v>60</v>
+      </c>
+      <c r="D26" s="49" t="n">
         <f aca="false">F26/0.0254</f>
         <v>0.0393700787401575</v>
       </c>
       <c r="E26" s="29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F26" s="30" t="n">
         <v>0.001</v>
       </c>
       <c r="G26" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H26" s="29"/>
-      <c r="I26" s="46"/>
+      <c r="I26" s="47"/>
       <c r="K26" s="16"/>
-      <c r="L26" s="19"/>
-      <c r="M26" s="19"/>
-      <c r="N26" s="19"/>
-      <c r="O26" s="19"/>
-      <c r="P26" s="19"/>
-      <c r="Q26" s="19"/>
+      <c r="L26" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="M26" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="N26" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="O26" s="29" t="n">
+        <f aca="false">M26*6895</f>
+        <v>103425</v>
+      </c>
+      <c r="P26" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q26" s="29"/>
       <c r="R26" s="20"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="42"/>
+      <c r="B27" s="43"/>
       <c r="C27" s="29" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D27" s="29" t="n">
         <f aca="false">D25+D24-D23</f>
         <v>24</v>
       </c>
       <c r="E27" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F27" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F27" s="48" t="n">
         <f aca="false">D27*0.0254</f>
         <v>0.6096</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H27" s="29"/>
-      <c r="I27" s="46"/>
-      <c r="K27" s="49"/>
-      <c r="L27" s="50"/>
-      <c r="M27" s="50"/>
-      <c r="N27" s="50"/>
-      <c r="O27" s="50"/>
-      <c r="P27" s="50"/>
-      <c r="Q27" s="50"/>
-      <c r="R27" s="51"/>
+      <c r="I27" s="47"/>
+      <c r="K27" s="16"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="19"/>
+      <c r="N27" s="19"/>
+      <c r="O27" s="19"/>
+      <c r="P27" s="19"/>
+      <c r="Q27" s="19"/>
+      <c r="R27" s="20"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="42"/>
+      <c r="B28" s="43"/>
       <c r="C28" s="29" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D28" s="29" t="n">
         <f aca="false">D22-D23-D25-D24</f>
         <v>9</v>
       </c>
       <c r="E28" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F28" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F28" s="48" t="n">
         <f aca="false">D28*0.0254</f>
         <v>0.2286</v>
       </c>
       <c r="G28" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H28" s="29"/>
-      <c r="I28" s="46"/>
+      <c r="I28" s="47"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19"/>
+      <c r="N28" s="19"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="19"/>
+      <c r="Q28" s="19"/>
+      <c r="R28" s="20"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="42"/>
-      <c r="C29" s="45"/>
-      <c r="D29" s="45"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="45"/>
-      <c r="G29" s="45"/>
-      <c r="H29" s="45"/>
-      <c r="I29" s="46"/>
+      <c r="B29" s="43"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="46"/>
+      <c r="I29" s="47"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="19"/>
+      <c r="N29" s="19"/>
+      <c r="O29" s="19"/>
+      <c r="P29" s="19"/>
+      <c r="Q29" s="19"/>
+      <c r="R29" s="20"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="42"/>
-      <c r="C30" s="43" t="s">
-        <v>55</v>
-      </c>
-      <c r="D30" s="44"/>
-      <c r="E30" s="44"/>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="45"/>
-      <c r="I30" s="46"/>
+      <c r="B30" s="43"/>
+      <c r="C30" s="44" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30" s="45"/>
+      <c r="E30" s="45"/>
+      <c r="F30" s="45"/>
+      <c r="G30" s="45"/>
+      <c r="H30" s="46"/>
+      <c r="I30" s="47"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="19"/>
+      <c r="M30" s="19"/>
+      <c r="N30" s="19"/>
+      <c r="O30" s="19"/>
+      <c r="P30" s="19"/>
+      <c r="Q30" s="19"/>
+      <c r="R30" s="20"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="42"/>
+      <c r="B31" s="43"/>
       <c r="C31" s="29" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="D31" s="30" t="n">
         <v>12</v>
       </c>
       <c r="E31" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F31" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F31" s="48" t="n">
         <f aca="false">D31*0.0254</f>
         <v>0.3048</v>
       </c>
       <c r="G31" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H31" s="29"/>
-      <c r="I31" s="46"/>
+      <c r="I31" s="47"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="19"/>
+      <c r="N31" s="19"/>
+      <c r="O31" s="19"/>
+      <c r="P31" s="19"/>
+      <c r="Q31" s="19"/>
+      <c r="R31" s="20"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="42"/>
+      <c r="B32" s="43"/>
       <c r="C32" s="29" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D32" s="30" t="n">
         <v>0.3125</v>
       </c>
       <c r="E32" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F32" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F32" s="48" t="n">
         <f aca="false">D32*0.0254</f>
         <v>0.0079375</v>
       </c>
       <c r="G32" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H32" s="29"/>
-      <c r="I32" s="46"/>
+      <c r="I32" s="47"/>
+      <c r="K32" s="16"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="19"/>
+      <c r="N32" s="19"/>
+      <c r="O32" s="19"/>
+      <c r="P32" s="19"/>
+      <c r="Q32" s="19"/>
+      <c r="R32" s="20"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="42"/>
+      <c r="B33" s="43"/>
       <c r="C33" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="D33" s="52" t="n">
+        <v>67</v>
+      </c>
+      <c r="D33" s="50" t="n">
         <v>3.94E-006</v>
       </c>
       <c r="E33" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F33" s="53" t="n">
+        <v>46</v>
+      </c>
+      <c r="F33" s="51" t="n">
         <f aca="false">D33*0.0254</f>
         <v>1.00076E-007</v>
       </c>
       <c r="G33" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H33" s="29"/>
-      <c r="I33" s="46"/>
+      <c r="I33" s="47"/>
+      <c r="K33" s="16"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="19"/>
+      <c r="N33" s="19"/>
+      <c r="O33" s="19"/>
+      <c r="P33" s="19"/>
+      <c r="Q33" s="19"/>
+      <c r="R33" s="20"/>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="42"/>
+      <c r="B34" s="43"/>
       <c r="C34" s="29" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="D34" s="30" t="n">
         <v>48</v>
       </c>
       <c r="E34" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F34" s="54" t="n">
+        <v>46</v>
+      </c>
+      <c r="F34" s="42" t="n">
         <f aca="false">D34*0.0254</f>
         <v>1.2192</v>
       </c>
       <c r="G34" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H34" s="29"/>
-      <c r="I34" s="46"/>
+      <c r="I34" s="47"/>
+      <c r="K34" s="16"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="19"/>
+      <c r="N34" s="19"/>
+      <c r="O34" s="19"/>
+      <c r="P34" s="19"/>
+      <c r="Q34" s="19"/>
+      <c r="R34" s="20"/>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="42"/>
+      <c r="B35" s="43"/>
       <c r="C35" s="29" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D35" s="30" t="n">
         <v>0.225</v>
       </c>
       <c r="E35" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F35" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F35" s="48" t="n">
         <f aca="false">D35*0.0254</f>
         <v>0.005715</v>
       </c>
       <c r="G35" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H35" s="29"/>
-      <c r="I35" s="46"/>
+      <c r="I35" s="47"/>
+      <c r="K35" s="52"/>
+      <c r="L35" s="53"/>
+      <c r="M35" s="53"/>
+      <c r="N35" s="53"/>
+      <c r="O35" s="53"/>
+      <c r="P35" s="53"/>
+      <c r="Q35" s="53"/>
+      <c r="R35" s="54"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="42"/>
+      <c r="B36" s="43"/>
       <c r="C36" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="D36" s="52" t="n">
+        <v>70</v>
+      </c>
+      <c r="D36" s="50" t="n">
         <v>3.94E-006</v>
       </c>
       <c r="E36" s="29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F36" s="29" t="n">
         <f aca="false">D36*0.0254</f>
         <v>1.00076E-007</v>
       </c>
       <c r="G36" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H36" s="29"/>
-      <c r="I36" s="46"/>
+      <c r="I36" s="47"/>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="42"/>
-      <c r="C37" s="45"/>
-      <c r="D37" s="45"/>
-      <c r="E37" s="45"/>
-      <c r="F37" s="45"/>
-      <c r="G37" s="45"/>
-      <c r="H37" s="45"/>
-      <c r="I37" s="46"/>
+      <c r="B37" s="43"/>
+      <c r="C37" s="46"/>
+      <c r="D37" s="46"/>
+      <c r="E37" s="46"/>
+      <c r="F37" s="46"/>
+      <c r="G37" s="46"/>
+      <c r="H37" s="46"/>
+      <c r="I37" s="47"/>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="42"/>
-      <c r="C38" s="43" t="s">
-        <v>62</v>
-      </c>
-      <c r="D38" s="44"/>
-      <c r="E38" s="44"/>
-      <c r="F38" s="44"/>
-      <c r="G38" s="44"/>
-      <c r="H38" s="45"/>
-      <c r="I38" s="46"/>
+      <c r="B38" s="43"/>
+      <c r="C38" s="44" t="s">
+        <v>71</v>
+      </c>
+      <c r="D38" s="45"/>
+      <c r="E38" s="45"/>
+      <c r="F38" s="45"/>
+      <c r="G38" s="45"/>
+      <c r="H38" s="46"/>
+      <c r="I38" s="47"/>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="42"/>
+      <c r="B39" s="43"/>
       <c r="C39" s="29" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D39" s="30" t="n">
         <v>6</v>
       </c>
       <c r="E39" s="29"/>
-      <c r="F39" s="47"/>
+      <c r="F39" s="48"/>
       <c r="G39" s="29"/>
       <c r="H39" s="29"/>
-      <c r="I39" s="46"/>
+      <c r="I39" s="47"/>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="42"/>
+      <c r="B40" s="43"/>
       <c r="C40" s="29" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="D40" s="30" t="n">
         <v>0.089</v>
       </c>
       <c r="E40" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F40" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F40" s="48" t="n">
         <f aca="false">D40*0.0254</f>
         <v>0.0022606</v>
       </c>
       <c r="G40" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H40" s="29"/>
-      <c r="I40" s="46"/>
+      <c r="I40" s="47"/>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="42"/>
+      <c r="B41" s="43"/>
       <c r="C41" s="29" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="D41" s="30" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="E41" s="29"/>
       <c r="F41" s="29"/>
       <c r="G41" s="29"/>
       <c r="H41" s="29"/>
-      <c r="I41" s="46"/>
+      <c r="I41" s="47"/>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="42"/>
+      <c r="B42" s="43"/>
       <c r="C42" s="29" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="D42" s="30" t="n">
         <v>6</v>
@@ -1951,33 +2082,33 @@
       <c r="F42" s="29"/>
       <c r="G42" s="29"/>
       <c r="H42" s="29"/>
-      <c r="I42" s="46"/>
+      <c r="I42" s="47"/>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="42"/>
+      <c r="B43" s="43"/>
       <c r="C43" s="29" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="D43" s="30" t="n">
         <v>0.0469</v>
       </c>
       <c r="E43" s="29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F43" s="29" t="n">
         <f aca="false">D43*0.0254</f>
         <v>0.00119126</v>
       </c>
       <c r="G43" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H43" s="29"/>
-      <c r="I43" s="46"/>
+      <c r="I43" s="47"/>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="42"/>
+      <c r="B44" s="43"/>
       <c r="C44" s="29" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="D44" s="30" t="n">
         <v>0.55</v>
@@ -1986,202 +2117,202 @@
       <c r="F44" s="29"/>
       <c r="G44" s="29"/>
       <c r="H44" s="29"/>
-      <c r="I44" s="46"/>
+      <c r="I44" s="47"/>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="42"/>
-      <c r="C45" s="45"/>
-      <c r="D45" s="45"/>
-      <c r="E45" s="45"/>
-      <c r="F45" s="45"/>
-      <c r="G45" s="45"/>
-      <c r="H45" s="45"/>
-      <c r="I45" s="46"/>
+      <c r="B45" s="43"/>
+      <c r="C45" s="46"/>
+      <c r="D45" s="46"/>
+      <c r="E45" s="46"/>
+      <c r="F45" s="46"/>
+      <c r="G45" s="46"/>
+      <c r="H45" s="46"/>
+      <c r="I45" s="47"/>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="42"/>
-      <c r="C46" s="43" t="s">
-        <v>69</v>
-      </c>
-      <c r="D46" s="44"/>
-      <c r="E46" s="44"/>
-      <c r="F46" s="44"/>
-      <c r="G46" s="44"/>
-      <c r="H46" s="45"/>
-      <c r="I46" s="46"/>
+      <c r="B46" s="43"/>
+      <c r="C46" s="44" t="s">
+        <v>78</v>
+      </c>
+      <c r="D46" s="45"/>
+      <c r="E46" s="45"/>
+      <c r="F46" s="45"/>
+      <c r="G46" s="45"/>
+      <c r="H46" s="46"/>
+      <c r="I46" s="47"/>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="42"/>
+      <c r="B47" s="43"/>
       <c r="C47" s="29" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="D47" s="30" t="n">
         <v>2</v>
       </c>
       <c r="E47" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F47" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F47" s="48" t="n">
         <f aca="false">D47*0.0254</f>
         <v>0.0508</v>
       </c>
       <c r="G47" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H47" s="29"/>
-      <c r="I47" s="46"/>
+      <c r="I47" s="47"/>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="42"/>
+      <c r="B48" s="43"/>
       <c r="C48" s="29" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="D48" s="30" t="n">
         <v>0.25</v>
       </c>
       <c r="E48" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F48" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F48" s="48" t="n">
         <f aca="false">D48*0.0254</f>
         <v>0.00635</v>
       </c>
       <c r="G48" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H48" s="29"/>
-      <c r="I48" s="46"/>
+      <c r="I48" s="47"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="42"/>
+      <c r="B49" s="43"/>
       <c r="C49" s="29" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="D49" s="30" t="n">
         <v>5</v>
       </c>
       <c r="E49" s="29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F49" s="29" t="n">
         <f aca="false">D49*0.0254</f>
         <v>0.127</v>
       </c>
       <c r="G49" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H49" s="29"/>
-      <c r="I49" s="46"/>
+      <c r="I49" s="47"/>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="42"/>
-      <c r="C50" s="45"/>
-      <c r="D50" s="45"/>
-      <c r="E50" s="45"/>
-      <c r="F50" s="45"/>
-      <c r="G50" s="45"/>
-      <c r="H50" s="45"/>
-      <c r="I50" s="46"/>
+      <c r="B50" s="43"/>
+      <c r="C50" s="46"/>
+      <c r="D50" s="46"/>
+      <c r="E50" s="46"/>
+      <c r="F50" s="46"/>
+      <c r="G50" s="46"/>
+      <c r="H50" s="46"/>
+      <c r="I50" s="47"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="42"/>
-      <c r="C51" s="43" t="s">
-        <v>73</v>
-      </c>
-      <c r="D51" s="44"/>
-      <c r="E51" s="44"/>
-      <c r="F51" s="44"/>
-      <c r="G51" s="44"/>
-      <c r="H51" s="45"/>
-      <c r="I51" s="46"/>
+      <c r="B51" s="43"/>
+      <c r="C51" s="44" t="s">
+        <v>82</v>
+      </c>
+      <c r="D51" s="45"/>
+      <c r="E51" s="45"/>
+      <c r="F51" s="45"/>
+      <c r="G51" s="45"/>
+      <c r="H51" s="46"/>
+      <c r="I51" s="47"/>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="42"/>
+      <c r="B52" s="43"/>
       <c r="C52" s="29" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="D52" s="30" t="n">
         <v>1</v>
       </c>
       <c r="E52" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F52" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F52" s="48" t="n">
         <f aca="false">D52*0.0254</f>
         <v>0.0254</v>
       </c>
       <c r="G52" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H52" s="29"/>
-      <c r="I52" s="46"/>
+      <c r="I52" s="47"/>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="42"/>
+      <c r="B53" s="43"/>
       <c r="C53" s="29" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="D53" s="30" t="n">
         <v>2</v>
       </c>
       <c r="E53" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F53" s="47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F53" s="48" t="n">
         <f aca="false">D53*0.0254</f>
         <v>0.0508</v>
       </c>
       <c r="G53" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H53" s="29"/>
-      <c r="I53" s="46"/>
+      <c r="I53" s="47"/>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="42"/>
+      <c r="B54" s="43"/>
       <c r="C54" s="29" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="D54" s="30" t="n">
         <v>15</v>
       </c>
       <c r="E54" s="29" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="F54" s="29"/>
       <c r="G54" s="29"/>
       <c r="H54" s="29"/>
-      <c r="I54" s="46"/>
+      <c r="I54" s="47"/>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="42"/>
-      <c r="C55" s="45"/>
-      <c r="D55" s="45"/>
-      <c r="E55" s="45"/>
-      <c r="F55" s="45"/>
-      <c r="G55" s="45"/>
-      <c r="H55" s="45"/>
-      <c r="I55" s="46"/>
+      <c r="B55" s="43"/>
+      <c r="C55" s="46"/>
+      <c r="D55" s="46"/>
+      <c r="E55" s="46"/>
+      <c r="F55" s="46"/>
+      <c r="G55" s="46"/>
+      <c r="H55" s="46"/>
+      <c r="I55" s="47"/>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="42"/>
-      <c r="C56" s="45"/>
-      <c r="D56" s="45"/>
-      <c r="E56" s="45"/>
-      <c r="F56" s="45"/>
-      <c r="G56" s="45"/>
-      <c r="H56" s="45"/>
-      <c r="I56" s="46"/>
+      <c r="B56" s="43"/>
+      <c r="C56" s="46"/>
+      <c r="D56" s="46"/>
+      <c r="E56" s="46"/>
+      <c r="F56" s="46"/>
+      <c r="G56" s="46"/>
+      <c r="H56" s="46"/>
+      <c r="I56" s="47"/>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="42"/>
-      <c r="C57" s="45"/>
-      <c r="D57" s="45"/>
-      <c r="E57" s="45"/>
-      <c r="F57" s="45"/>
-      <c r="G57" s="45"/>
-      <c r="H57" s="45"/>
-      <c r="I57" s="46"/>
+      <c r="B57" s="43"/>
+      <c r="C57" s="46"/>
+      <c r="D57" s="46"/>
+      <c r="E57" s="46"/>
+      <c r="F57" s="46"/>
+      <c r="G57" s="46"/>
+      <c r="H57" s="46"/>
+      <c r="I57" s="47"/>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="55"/>
@@ -2222,8 +2353,8 @@
       <formula1>"0,1"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F6:F7" type="none">
-      <formula1>"Isopropanol","Ethanol","E98","E85"</formula1>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="F6:F7" type="none">
+      <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2250,22 +2381,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2275,127 +2406,127 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2410,37 +2541,37 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Input sheet: replace ambient temperature with nitrous temperature as the input
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="89">
   <si>
     <t xml:space="preserve">SIMULATION SETUP</t>
   </si>
@@ -104,187 +104,190 @@
     <t xml:space="preserve">C* Efficiency</t>
   </si>
   <si>
+    <t xml:space="preserve">Nitrous Temperature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambient – 10deg F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nozzle Efficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambient Pressure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">psi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambient at FAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decay Constant (liquid)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decay Constant (vapor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GEOMETRIC CHARACTERISTICS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feed System ΔP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ball Valve Cv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Ball Valve K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tank OD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Ball Valve K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tank Wall Thickness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer No. Elbows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tank Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel No. Elbows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulkhead Insertion Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrance K-factor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piston Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elbow K-factor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Static Vent Position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measured from tank aft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Sum K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Static Vent Diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Sum K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Piston Loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feed System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Line Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Line Diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Line Roughness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Line Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Line Diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Line Roughness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Injector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Oxidizer Holes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Hole Diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxidizer Cd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Fuel Holes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Hole Diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Cd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamber </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamber ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamber Wall Thickness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chamber Length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nozzle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Throat Diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exit Diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exit Half Angle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">deg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sweepable parameters (dropdown source for the sweep block)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ambient Temperature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nozzle Efficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nitrous Temperature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decay Constant (liquid)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambient Pressure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">psi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambient at FAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decay Constant (vapor)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1/s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feed System ΔP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GEOMETRIC CHARACTERISTICS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ball Valve Cv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oxidizer Ball Valve K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Ball Valve K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tank OD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oxidizer No. Elbows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tank Wall Thickness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel No. Elbows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tank Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entrance K-factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bulkhead Insertion Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elbow K-factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Piston Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oxidizer Sum K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Static Vent Position</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Measured from tank aft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Sum K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Static Vent Diameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Piston Loss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oxidizer Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feed System</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oxidizer Line Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oxidizer Line Diameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oxidizer Line Roughness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Line Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Line Diameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Line Roughness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Injector</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No. Oxidizer Holes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oxidizer Hole Diameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oxidizer Cd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No. Fuel Holes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Hole Diameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Cd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chamber </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chamber ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chamber Wall Thickness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chamber Length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nozzle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Throat Diameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exit Diameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exit Half Angle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sweepable parameters (dropdown source for the sweep block)</t>
   </si>
 </sst>
 </file>
@@ -484,7 +487,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -621,6 +624,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -653,27 +660,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1027,7 +1034,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:R58"/>
+  <dimension ref="B2:R57"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="3.24"/>
@@ -1299,24 +1306,26 @@
       <c r="C12" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="30" t="n">
-        <v>60</v>
+      <c r="D12" s="34" t="n">
+        <v>50</v>
       </c>
       <c r="E12" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="F12" s="34" t="n">
+      <c r="F12" s="35" t="n">
         <f aca="false">(D12-32)/1.8</f>
-        <v>15.5555555555556</v>
+        <v>10</v>
       </c>
       <c r="G12" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="H12" s="29"/>
+      <c r="H12" s="29" t="s">
+        <v>30</v>
+      </c>
       <c r="I12" s="15"/>
       <c r="K12" s="16"/>
       <c r="L12" s="29" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M12" s="30" t="n">
         <v>0.95</v>
@@ -1330,27 +1339,28 @@
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="11"/>
       <c r="C13" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="29" t="n">
-        <f aca="false">D12-10</f>
-        <v>50</v>
+        <v>32</v>
+      </c>
+      <c r="D13" s="30" t="n">
+        <v>13.5</v>
       </c>
       <c r="E13" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="F13" s="34" t="n">
-        <f aca="false">(D13-32)/1.8</f>
-        <v>10</v>
+        <v>33</v>
+      </c>
+      <c r="F13" s="29" t="n">
+        <f aca="false">D13*6895</f>
+        <v>93082.5</v>
       </c>
       <c r="G13" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="H13" s="29"/>
+        <v>34</v>
+      </c>
+      <c r="H13" s="29" t="s">
+        <v>35</v>
+      </c>
       <c r="I13" s="15"/>
       <c r="K13" s="16"/>
       <c r="L13" s="29" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="M13" s="30" t="n">
         <v>0.7</v>
@@ -1362,27 +1372,14 @@
       <c r="R13" s="20"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="11"/>
-      <c r="C14" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="30" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="E14" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="F14" s="29" t="n">
-        <f aca="false">D14*6895</f>
-        <v>93082.5</v>
-      </c>
-      <c r="G14" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="H14" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="I14" s="15"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="38"/>
       <c r="K14" s="16"/>
       <c r="L14" s="29" t="s">
         <v>37</v>
@@ -1399,14 +1396,6 @@
       <c r="R14" s="20"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="35"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="37"/>
       <c r="K15" s="16"/>
       <c r="L15" s="33"/>
       <c r="M15" s="33"/>
@@ -1417,9 +1406,12 @@
       <c r="R15" s="20"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="K16" s="16"/>
       <c r="L16" s="32" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M16" s="33"/>
       <c r="N16" s="33"/>
@@ -1429,9 +1421,14 @@
       <c r="R16" s="20"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="2" t="s">
-        <v>40</v>
-      </c>
+      <c r="B17" s="39"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="42"/>
       <c r="K17" s="16"/>
       <c r="L17" s="29" t="s">
         <v>41</v>
@@ -1446,20 +1443,22 @@
       <c r="R17" s="20"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="38"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="41"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="44" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18" s="45"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="45"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="47"/>
       <c r="K18" s="16"/>
       <c r="L18" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="M18" s="42" t="n">
-        <f aca="false">891 * D32^4 / M17^2</f>
+        <v>43</v>
+      </c>
+      <c r="M18" s="48" t="n">
+        <f aca="false">891 * D31^4 / M17^2</f>
         <v>3.31923365592957</v>
       </c>
       <c r="N18" s="29"/>
@@ -1470,21 +1469,30 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="43"/>
-      <c r="C19" s="44" t="s">
-        <v>43</v>
-      </c>
-      <c r="D19" s="45"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="46"/>
+      <c r="C19" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F19" s="49" t="n">
+        <f aca="false">D19*0.0254</f>
+        <v>0.1016</v>
+      </c>
+      <c r="G19" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="H19" s="29"/>
       <c r="I19" s="47"/>
       <c r="K19" s="16"/>
       <c r="L19" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="M19" s="42" t="n">
-        <f aca="false">891 * D35^4 / M17^2</f>
+        <v>47</v>
+      </c>
+      <c r="M19" s="48" t="n">
+        <f aca="false">891 * D34^4 / M17^2</f>
         <v>0.892006072998047</v>
       </c>
       <c r="N19" s="29"/>
@@ -1496,26 +1504,26 @@
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="43"/>
       <c r="C20" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="30" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="E20" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="D20" s="30" t="n">
-        <v>4</v>
-      </c>
-      <c r="E20" s="29" t="s">
+      <c r="F20" s="49" t="n">
+        <f aca="false">D20*0.0254</f>
+        <v>0.003175</v>
+      </c>
+      <c r="G20" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F20" s="48" t="n">
-        <f aca="false">D20*0.0254</f>
-        <v>0.1016</v>
-      </c>
-      <c r="G20" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H20" s="29"/>
       <c r="I20" s="47"/>
       <c r="K20" s="16"/>
       <c r="L20" s="29" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M20" s="30" t="n">
         <v>0</v>
@@ -1529,26 +1537,26 @@
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="43"/>
       <c r="C21" s="29" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D21" s="30" t="n">
-        <v>0.125</v>
+        <v>36</v>
       </c>
       <c r="E21" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F21" s="49" t="n">
+        <f aca="false">D21*0.0254</f>
+        <v>0.9144</v>
+      </c>
+      <c r="G21" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F21" s="48" t="n">
-        <f aca="false">D21*0.0254</f>
-        <v>0.003175</v>
-      </c>
-      <c r="G21" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H21" s="29"/>
       <c r="I21" s="47"/>
       <c r="K21" s="16"/>
       <c r="L21" s="29" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M21" s="30" t="n">
         <v>2</v>
@@ -1562,26 +1570,26 @@
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="43"/>
       <c r="C22" s="29" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D22" s="30" t="n">
-        <v>36</v>
+        <v>1.5</v>
       </c>
       <c r="E22" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F22" s="49" t="n">
+        <f aca="false">D22*0.0254</f>
+        <v>0.0381</v>
+      </c>
+      <c r="G22" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F22" s="48" t="n">
-        <f aca="false">D22*0.0254</f>
-        <v>0.9144</v>
-      </c>
-      <c r="G22" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H22" s="29"/>
       <c r="I22" s="47"/>
       <c r="K22" s="16"/>
       <c r="L22" s="29" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M22" s="30" t="n">
         <v>0.5</v>
@@ -1595,26 +1603,26 @@
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="43"/>
       <c r="C23" s="29" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D23" s="30" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="E23" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F23" s="49" t="n">
+        <f aca="false">D23*0.0254</f>
+        <v>0.0762</v>
+      </c>
+      <c r="G23" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F23" s="48" t="n">
-        <f aca="false">D23*0.0254</f>
-        <v>0.0381</v>
-      </c>
-      <c r="G23" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H23" s="29"/>
       <c r="I23" s="47"/>
       <c r="K23" s="16"/>
       <c r="L23" s="29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M23" s="30" t="n">
         <v>0.8</v>
@@ -1628,28 +1636,30 @@
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="43"/>
       <c r="C24" s="29" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D24" s="30" t="n">
-        <v>3</v>
+        <v>22.5</v>
       </c>
       <c r="E24" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F24" s="49" t="n">
+        <f aca="false">D24*0.0254</f>
+        <v>0.5715</v>
+      </c>
+      <c r="G24" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="F24" s="48" t="n">
-        <f aca="false">D24*0.0254</f>
-        <v>0.0762</v>
-      </c>
-      <c r="G24" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="H24" s="29"/>
+      <c r="H24" s="29" t="s">
+        <v>57</v>
+      </c>
       <c r="I24" s="47"/>
       <c r="K24" s="16"/>
       <c r="L24" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="M24" s="42" t="n">
+        <v>58</v>
+      </c>
+      <c r="M24" s="48" t="n">
         <f aca="false">M23*M20+M18 + M22</f>
         <v>3.81923365592957</v>
       </c>
@@ -1662,30 +1672,28 @@
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="43"/>
       <c r="C25" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="D25" s="30" t="n">
-        <v>22.5</v>
+        <v>59</v>
+      </c>
+      <c r="D25" s="50" t="n">
+        <f aca="false">F25/0.0254</f>
+        <v>0.0393700787401575</v>
       </c>
       <c r="E25" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F25" s="30" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G25" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="F25" s="48" t="n">
-        <f aca="false">D25*0.0254</f>
-        <v>0.5715</v>
-      </c>
-      <c r="G25" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="H25" s="29" t="s">
-        <v>58</v>
-      </c>
+      <c r="H25" s="29"/>
       <c r="I25" s="47"/>
       <c r="K25" s="16"/>
       <c r="L25" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="M25" s="42" t="n">
+        <v>60</v>
+      </c>
+      <c r="M25" s="48" t="n">
         <f aca="false">M19 + M23*M21 + M22</f>
         <v>2.99200607299805</v>
       </c>
@@ -1698,39 +1706,40 @@
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="43"/>
       <c r="C26" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="D26" s="49" t="n">
-        <f aca="false">F26/0.0254</f>
-        <v>0.0393700787401575</v>
+        <v>61</v>
+      </c>
+      <c r="D26" s="29" t="n">
+        <f aca="false">D24+D23-D22</f>
+        <v>24</v>
       </c>
       <c r="E26" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F26" s="49" t="n">
+        <f aca="false">D26*0.0254</f>
+        <v>0.6096</v>
+      </c>
+      <c r="G26" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F26" s="30" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G26" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H26" s="29"/>
       <c r="I26" s="47"/>
       <c r="K26" s="16"/>
       <c r="L26" s="29" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M26" s="30" t="n">
         <v>15</v>
       </c>
       <c r="N26" s="29" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O26" s="29" t="n">
         <f aca="false">M26*6895</f>
         <v>103425</v>
       </c>
       <c r="P26" s="29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Q26" s="29"/>
       <c r="R26" s="20"/>
@@ -1738,21 +1747,21 @@
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="43"/>
       <c r="C27" s="29" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D27" s="29" t="n">
-        <f aca="false">D25+D24-D23</f>
-        <v>24</v>
+        <f aca="false">D21-D22-D24-D23</f>
+        <v>9</v>
       </c>
       <c r="E27" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F27" s="49" t="n">
+        <f aca="false">D27*0.0254</f>
+        <v>0.2286</v>
+      </c>
+      <c r="G27" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F27" s="48" t="n">
-        <f aca="false">D27*0.0254</f>
-        <v>0.6096</v>
-      </c>
-      <c r="G27" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H27" s="29"/>
       <c r="I27" s="47"/>
@@ -1767,24 +1776,12 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="43"/>
-      <c r="C28" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="D28" s="29" t="n">
-        <f aca="false">D22-D23-D25-D24</f>
-        <v>9</v>
-      </c>
-      <c r="E28" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="F28" s="48" t="n">
-        <f aca="false">D28*0.0254</f>
-        <v>0.2286</v>
-      </c>
-      <c r="G28" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="H28" s="29"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="46"/>
       <c r="I28" s="47"/>
       <c r="K28" s="16"/>
       <c r="L28" s="19"/>
@@ -1797,11 +1794,13 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="43"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="46"/>
+      <c r="C29" s="44" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" s="45"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="45"/>
+      <c r="G29" s="45"/>
       <c r="H29" s="46"/>
       <c r="I29" s="47"/>
       <c r="K29" s="16"/>
@@ -1815,14 +1814,23 @@
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="43"/>
-      <c r="C30" s="44" t="s">
-        <v>64</v>
-      </c>
-      <c r="D30" s="45"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="45"/>
-      <c r="G30" s="45"/>
-      <c r="H30" s="46"/>
+      <c r="C30" s="29" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="E30" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F30" s="49" t="n">
+        <f aca="false">D30*0.0254</f>
+        <v>0.3048</v>
+      </c>
+      <c r="G30" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="H30" s="29"/>
       <c r="I30" s="47"/>
       <c r="K30" s="16"/>
       <c r="L30" s="19"/>
@@ -1836,20 +1844,20 @@
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="43"/>
       <c r="C31" s="29" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D31" s="30" t="n">
-        <v>12</v>
+        <v>0.3125</v>
       </c>
       <c r="E31" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F31" s="49" t="n">
+        <f aca="false">D31*0.0254</f>
+        <v>0.0079375</v>
+      </c>
+      <c r="G31" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F31" s="48" t="n">
-        <f aca="false">D31*0.0254</f>
-        <v>0.3048</v>
-      </c>
-      <c r="G31" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H31" s="29"/>
       <c r="I31" s="47"/>
@@ -1865,20 +1873,20 @@
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="43"/>
       <c r="C32" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="D32" s="30" t="n">
-        <v>0.3125</v>
+        <v>67</v>
+      </c>
+      <c r="D32" s="51" t="n">
+        <v>3.94E-006</v>
       </c>
       <c r="E32" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F32" s="52" t="n">
+        <f aca="false">D32*0.0254</f>
+        <v>1.00076E-007</v>
+      </c>
+      <c r="G32" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F32" s="48" t="n">
-        <f aca="false">D32*0.0254</f>
-        <v>0.0079375</v>
-      </c>
-      <c r="G32" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H32" s="29"/>
       <c r="I32" s="47"/>
@@ -1894,20 +1902,20 @@
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="43"/>
       <c r="C33" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="D33" s="50" t="n">
-        <v>3.94E-006</v>
+        <v>68</v>
+      </c>
+      <c r="D33" s="30" t="n">
+        <v>48</v>
       </c>
       <c r="E33" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F33" s="48" t="n">
+        <f aca="false">D33*0.0254</f>
+        <v>1.2192</v>
+      </c>
+      <c r="G33" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F33" s="51" t="n">
-        <f aca="false">D33*0.0254</f>
-        <v>1.00076E-007</v>
-      </c>
-      <c r="G33" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H33" s="29"/>
       <c r="I33" s="47"/>
@@ -1923,20 +1931,20 @@
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="43"/>
       <c r="C34" s="29" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D34" s="30" t="n">
-        <v>48</v>
+        <v>0.225</v>
       </c>
       <c r="E34" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F34" s="49" t="n">
+        <f aca="false">D34*0.0254</f>
+        <v>0.005715</v>
+      </c>
+      <c r="G34" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F34" s="42" t="n">
-        <f aca="false">D34*0.0254</f>
-        <v>1.2192</v>
-      </c>
-      <c r="G34" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H34" s="29"/>
       <c r="I34" s="47"/>
@@ -1952,117 +1960,110 @@
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="43"/>
       <c r="C35" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="D35" s="30" t="n">
-        <v>0.225</v>
+        <v>70</v>
+      </c>
+      <c r="D35" s="51" t="n">
+        <v>3.94E-006</v>
       </c>
       <c r="E35" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F35" s="29" t="n">
+        <f aca="false">D35*0.0254</f>
+        <v>1.00076E-007</v>
+      </c>
+      <c r="G35" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F35" s="48" t="n">
-        <f aca="false">D35*0.0254</f>
-        <v>0.005715</v>
-      </c>
-      <c r="G35" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H35" s="29"/>
       <c r="I35" s="47"/>
-      <c r="K35" s="52"/>
-      <c r="L35" s="53"/>
-      <c r="M35" s="53"/>
-      <c r="N35" s="53"/>
-      <c r="O35" s="53"/>
-      <c r="P35" s="53"/>
-      <c r="Q35" s="53"/>
-      <c r="R35" s="54"/>
+      <c r="K35" s="53"/>
+      <c r="L35" s="54"/>
+      <c r="M35" s="54"/>
+      <c r="N35" s="54"/>
+      <c r="O35" s="54"/>
+      <c r="P35" s="54"/>
+      <c r="Q35" s="54"/>
+      <c r="R35" s="55"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="43"/>
-      <c r="C36" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="D36" s="50" t="n">
-        <v>3.94E-006</v>
-      </c>
-      <c r="E36" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="F36" s="29" t="n">
-        <f aca="false">D36*0.0254</f>
-        <v>1.00076E-007</v>
-      </c>
-      <c r="G36" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="H36" s="29"/>
+      <c r="C36" s="46"/>
+      <c r="D36" s="46"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="46"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="46"/>
       <c r="I36" s="47"/>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="43"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="46"/>
-      <c r="E37" s="46"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="46"/>
+      <c r="C37" s="44" t="s">
+        <v>71</v>
+      </c>
+      <c r="D37" s="45"/>
+      <c r="E37" s="45"/>
+      <c r="F37" s="45"/>
+      <c r="G37" s="45"/>
       <c r="H37" s="46"/>
       <c r="I37" s="47"/>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="43"/>
-      <c r="C38" s="44" t="s">
-        <v>71</v>
-      </c>
-      <c r="D38" s="45"/>
-      <c r="E38" s="45"/>
-      <c r="F38" s="45"/>
-      <c r="G38" s="45"/>
-      <c r="H38" s="46"/>
+      <c r="C38" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="D38" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="E38" s="29"/>
+      <c r="F38" s="49"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="29"/>
       <c r="I38" s="47"/>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="43"/>
       <c r="C39" s="29" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D39" s="30" t="n">
-        <v>6</v>
-      </c>
-      <c r="E39" s="29"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="29"/>
+        <v>0.089</v>
+      </c>
+      <c r="E39" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F39" s="49" t="n">
+        <f aca="false">D39*0.0254</f>
+        <v>0.0022606</v>
+      </c>
+      <c r="G39" s="29" t="s">
+        <v>46</v>
+      </c>
       <c r="H39" s="29"/>
       <c r="I39" s="47"/>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="43"/>
       <c r="C40" s="29" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D40" s="30" t="n">
-        <v>0.089</v>
-      </c>
-      <c r="E40" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="F40" s="48" t="n">
-        <f aca="false">D40*0.0254</f>
-        <v>0.0022606</v>
-      </c>
-      <c r="G40" s="29" t="s">
-        <v>47</v>
-      </c>
+        <v>0.7</v>
+      </c>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
       <c r="H40" s="29"/>
       <c r="I40" s="47"/>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="43"/>
       <c r="C41" s="29" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D41" s="30" t="n">
-        <v>0.7</v>
+        <v>6</v>
       </c>
       <c r="E41" s="29"/>
       <c r="F41" s="29"/>
@@ -2073,91 +2074,98 @@
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="43"/>
       <c r="C42" s="29" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D42" s="30" t="n">
-        <v>6</v>
-      </c>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
+        <v>0.0469</v>
+      </c>
+      <c r="E42" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F42" s="29" t="n">
+        <f aca="false">D42*0.0254</f>
+        <v>0.00119126</v>
+      </c>
+      <c r="G42" s="29" t="s">
+        <v>46</v>
+      </c>
       <c r="H42" s="29"/>
       <c r="I42" s="47"/>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="43"/>
       <c r="C43" s="29" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D43" s="30" t="n">
-        <v>0.0469</v>
-      </c>
-      <c r="E43" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="F43" s="29" t="n">
-        <f aca="false">D43*0.0254</f>
-        <v>0.00119126</v>
-      </c>
-      <c r="G43" s="29" t="s">
-        <v>47</v>
-      </c>
+        <v>0.55</v>
+      </c>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
       <c r="H43" s="29"/>
       <c r="I43" s="47"/>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="43"/>
-      <c r="C44" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D44" s="30" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E44" s="29"/>
-      <c r="F44" s="29"/>
-      <c r="G44" s="29"/>
-      <c r="H44" s="29"/>
+      <c r="C44" s="46"/>
+      <c r="D44" s="46"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="46"/>
+      <c r="H44" s="46"/>
       <c r="I44" s="47"/>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="43"/>
-      <c r="C45" s="46"/>
-      <c r="D45" s="46"/>
-      <c r="E45" s="46"/>
-      <c r="F45" s="46"/>
-      <c r="G45" s="46"/>
+      <c r="C45" s="44" t="s">
+        <v>78</v>
+      </c>
+      <c r="D45" s="45"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
       <c r="H45" s="46"/>
       <c r="I45" s="47"/>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="43"/>
-      <c r="C46" s="44" t="s">
-        <v>78</v>
-      </c>
-      <c r="D46" s="45"/>
-      <c r="E46" s="45"/>
-      <c r="F46" s="45"/>
-      <c r="G46" s="45"/>
-      <c r="H46" s="46"/>
+      <c r="C46" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="D46" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F46" s="49" t="n">
+        <f aca="false">D46*0.0254</f>
+        <v>0.0508</v>
+      </c>
+      <c r="G46" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="H46" s="29"/>
       <c r="I46" s="47"/>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="43"/>
       <c r="C47" s="29" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D47" s="30" t="n">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="E47" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F47" s="49" t="n">
+        <f aca="false">D47*0.0254</f>
+        <v>0.00635</v>
+      </c>
+      <c r="G47" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F47" s="48" t="n">
-        <f aca="false">D47*0.0254</f>
-        <v>0.0508</v>
-      </c>
-      <c r="G47" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H47" s="29"/>
       <c r="I47" s="47"/>
@@ -2165,84 +2173,84 @@
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="43"/>
       <c r="C48" s="29" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D48" s="30" t="n">
-        <v>0.25</v>
+        <v>5</v>
       </c>
       <c r="E48" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F48" s="29" t="n">
+        <f aca="false">D48*0.0254</f>
+        <v>0.127</v>
+      </c>
+      <c r="G48" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F48" s="48" t="n">
-        <f aca="false">D48*0.0254</f>
-        <v>0.00635</v>
-      </c>
-      <c r="G48" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H48" s="29"/>
       <c r="I48" s="47"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="43"/>
-      <c r="C49" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="D49" s="30" t="n">
-        <v>5</v>
-      </c>
-      <c r="E49" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="F49" s="29" t="n">
-        <f aca="false">D49*0.0254</f>
-        <v>0.127</v>
-      </c>
-      <c r="G49" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="H49" s="29"/>
+      <c r="C49" s="46"/>
+      <c r="D49" s="46"/>
+      <c r="E49" s="46"/>
+      <c r="F49" s="46"/>
+      <c r="G49" s="46"/>
+      <c r="H49" s="46"/>
       <c r="I49" s="47"/>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="43"/>
-      <c r="C50" s="46"/>
-      <c r="D50" s="46"/>
-      <c r="E50" s="46"/>
-      <c r="F50" s="46"/>
-      <c r="G50" s="46"/>
+      <c r="C50" s="44" t="s">
+        <v>82</v>
+      </c>
+      <c r="D50" s="45"/>
+      <c r="E50" s="45"/>
+      <c r="F50" s="45"/>
+      <c r="G50" s="45"/>
       <c r="H50" s="46"/>
       <c r="I50" s="47"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="43"/>
-      <c r="C51" s="44" t="s">
-        <v>82</v>
-      </c>
-      <c r="D51" s="45"/>
-      <c r="E51" s="45"/>
-      <c r="F51" s="45"/>
-      <c r="G51" s="45"/>
-      <c r="H51" s="46"/>
+      <c r="C51" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="D51" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F51" s="49" t="n">
+        <f aca="false">D51*0.0254</f>
+        <v>0.0254</v>
+      </c>
+      <c r="G51" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="H51" s="29"/>
       <c r="I51" s="47"/>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="43"/>
       <c r="C52" s="29" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D52" s="30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F52" s="49" t="n">
+        <f aca="false">D52*0.0254</f>
+        <v>0.0508</v>
+      </c>
+      <c r="G52" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="F52" s="48" t="n">
-        <f aca="false">D52*0.0254</f>
-        <v>0.0254</v>
-      </c>
-      <c r="G52" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="H52" s="29"/>
       <c r="I52" s="47"/>
@@ -2250,38 +2258,27 @@
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="43"/>
       <c r="C53" s="29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D53" s="30" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E53" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="F53" s="48" t="n">
-        <f aca="false">D53*0.0254</f>
-        <v>0.0508</v>
-      </c>
-      <c r="G53" s="29" t="s">
-        <v>47</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="F53" s="29"/>
+      <c r="G53" s="29"/>
       <c r="H53" s="29"/>
       <c r="I53" s="47"/>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="43"/>
-      <c r="C54" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="D54" s="30" t="n">
-        <v>15</v>
-      </c>
-      <c r="E54" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="F54" s="29"/>
-      <c r="G54" s="29"/>
-      <c r="H54" s="29"/>
+      <c r="C54" s="46"/>
+      <c r="D54" s="46"/>
+      <c r="E54" s="46"/>
+      <c r="F54" s="46"/>
+      <c r="G54" s="46"/>
+      <c r="H54" s="46"/>
       <c r="I54" s="47"/>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2305,24 +2302,14 @@
       <c r="I56" s="47"/>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="43"/>
-      <c r="C57" s="46"/>
-      <c r="D57" s="46"/>
-      <c r="E57" s="46"/>
-      <c r="F57" s="46"/>
-      <c r="G57" s="46"/>
-      <c r="H57" s="46"/>
-      <c r="I57" s="47"/>
-    </row>
-    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="55"/>
-      <c r="C58" s="56"/>
-      <c r="D58" s="56"/>
-      <c r="E58" s="56"/>
-      <c r="F58" s="56"/>
-      <c r="G58" s="56"/>
-      <c r="H58" s="56"/>
-      <c r="I58" s="57"/>
+      <c r="B57" s="56"/>
+      <c r="C57" s="57"/>
+      <c r="D57" s="57"/>
+      <c r="E57" s="57"/>
+      <c r="F57" s="57"/>
+      <c r="G57" s="57"/>
+      <c r="H57" s="57"/>
+      <c r="I57" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -2337,8 +2324,8 @@
     <mergeCell ref="O5:P5"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="F9:G9"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M4" type="list">
@@ -2396,47 +2383,47 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>27</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2546,12 +2533,12 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2561,17 +2548,17 @@
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sweep list: Ambient Temperature -> Nitrous Temperature
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="88">
   <si>
     <t xml:space="preserve">SIMULATION SETUP</t>
   </si>
@@ -285,9 +285,6 @@
   </si>
   <si>
     <t xml:space="preserve">Sweepable parameters (dropdown source for the sweep block)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambient Temperature</t>
   </si>
 </sst>
 </file>
@@ -2383,7 +2380,7 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>88</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Dark mode for plots (THEME setting); input sheet updates
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="88">
   <si>
     <t xml:space="preserve">SIMULATION SETUP</t>
   </si>
@@ -65,6 +65,9 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
+    <t xml:space="preserve">No. Oxidizer Holes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fuel Density</t>
   </si>
   <si>
@@ -74,6 +77,9 @@
     <t xml:space="preserve">kg/m3</t>
   </si>
   <si>
+    <t xml:space="preserve">No. Fuel Holes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fuel Dynamic Viscosity</t>
   </si>
   <si>
@@ -239,16 +245,10 @@
     <t xml:space="preserve">Injector</t>
   </si>
   <si>
-    <t xml:space="preserve">No. Oxidizer Holes</t>
-  </si>
-  <si>
     <t xml:space="preserve">Oxidizer Hole Diameter</t>
   </si>
   <si>
     <t xml:space="preserve">Oxidizer Cd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No. Fuel Holes</t>
   </si>
   <si>
     <t xml:space="preserve">Fuel Hole Diameter</t>
@@ -1135,49 +1135,71 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="11"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="28"/>
+      <c r="C6" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" s="28" t="n">
+        <v>1</v>
+      </c>
       <c r="G6" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="21"/>
+      <c r="H6" s="21" t="n">
+        <f aca="false">(E6-D6)/F6</f>
+        <v>4</v>
+      </c>
       <c r="I6" s="15"/>
       <c r="K6" s="16"/>
       <c r="L6" s="29" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M6" s="29" t="n">
         <f aca="false">O6/16.0185</f>
         <v>49.0682648188033</v>
       </c>
       <c r="N6" s="29" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="O6" s="30" t="n">
         <v>786</v>
       </c>
       <c r="P6" s="29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q6" s="29"/>
       <c r="R6" s="20"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="11"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="28"/>
+      <c r="C7" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" s="28" t="n">
+        <v>1</v>
+      </c>
       <c r="G7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="21" t="n">
+        <f aca="false">(E7-D7)/F7</f>
+        <v>4</v>
+      </c>
       <c r="I7" s="15"/>
       <c r="K7" s="16"/>
       <c r="L7" s="29" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="M7" s="29"/>
       <c r="N7" s="29"/>
@@ -1185,7 +1207,7 @@
         <v>2.5</v>
       </c>
       <c r="P7" s="29" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="Q7" s="29"/>
       <c r="R7" s="20"/>
@@ -1193,7 +1215,7 @@
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="11"/>
       <c r="C8" s="12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D8" s="31"/>
       <c r="E8" s="31"/>
@@ -1203,7 +1225,7 @@
       <c r="I8" s="15"/>
       <c r="K8" s="16"/>
       <c r="L8" s="29" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M8" s="29"/>
       <c r="N8" s="29"/>
@@ -1211,10 +1233,10 @@
         <v>0.07</v>
       </c>
       <c r="P8" s="29" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="Q8" s="29" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="R8" s="20"/>
     </row>
@@ -1247,13 +1269,13 @@
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="11"/>
       <c r="C10" s="29" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D10" s="30" t="n">
         <v>0.01</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F10" s="29"/>
       <c r="G10" s="29"/>
@@ -1261,7 +1283,7 @@
       <c r="I10" s="15"/>
       <c r="K10" s="16"/>
       <c r="L10" s="32" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="M10" s="33"/>
       <c r="N10" s="33"/>
@@ -1273,13 +1295,13 @@
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="11"/>
       <c r="C11" s="29" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D11" s="30" t="n">
         <v>30</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F11" s="29"/>
       <c r="G11" s="29"/>
@@ -1287,7 +1309,7 @@
       <c r="I11" s="15"/>
       <c r="K11" s="16"/>
       <c r="L11" s="29" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="M11" s="30" t="n">
         <v>0.65</v>
@@ -1301,28 +1323,28 @@
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="11"/>
       <c r="C12" s="29" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D12" s="34" t="n">
         <v>50</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F12" s="35" t="n">
         <f aca="false">(D12-32)/1.8</f>
         <v>10</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H12" s="29" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I12" s="15"/>
       <c r="K12" s="16"/>
       <c r="L12" s="29" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="M12" s="30" t="n">
         <v>0.95</v>
@@ -1336,28 +1358,28 @@
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="11"/>
       <c r="C13" s="29" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D13" s="30" t="n">
         <v>13.5</v>
       </c>
       <c r="E13" s="29" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F13" s="29" t="n">
         <f aca="false">D13*6895</f>
         <v>93082.5</v>
       </c>
       <c r="G13" s="29" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H13" s="29" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I13" s="15"/>
       <c r="K13" s="16"/>
       <c r="L13" s="29" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M13" s="30" t="n">
         <v>0.7</v>
@@ -1379,13 +1401,13 @@
       <c r="I14" s="38"/>
       <c r="K14" s="16"/>
       <c r="L14" s="29" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="M14" s="30" t="n">
         <v>0.25</v>
       </c>
       <c r="N14" s="29" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="O14" s="29"/>
       <c r="P14" s="29"/>
@@ -1404,11 +1426,11 @@
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K16" s="16"/>
       <c r="L16" s="32" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="M16" s="33"/>
       <c r="N16" s="33"/>
@@ -1428,7 +1450,7 @@
       <c r="I17" s="42"/>
       <c r="K17" s="16"/>
       <c r="L17" s="29" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="M17" s="30" t="n">
         <v>1.6</v>
@@ -1442,7 +1464,7 @@
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="43"/>
       <c r="C18" s="44" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D18" s="45"/>
       <c r="E18" s="45"/>
@@ -1452,7 +1474,7 @@
       <c r="I18" s="47"/>
       <c r="K18" s="16"/>
       <c r="L18" s="29" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M18" s="48" t="n">
         <f aca="false">891 * D31^4 / M17^2</f>
@@ -1467,26 +1489,26 @@
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="43"/>
       <c r="C19" s="29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D19" s="30" t="n">
         <v>4</v>
       </c>
       <c r="E19" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F19" s="49" t="n">
         <f aca="false">D19*0.0254</f>
         <v>0.1016</v>
       </c>
       <c r="G19" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H19" s="29"/>
       <c r="I19" s="47"/>
       <c r="K19" s="16"/>
       <c r="L19" s="29" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="M19" s="48" t="n">
         <f aca="false">891 * D34^4 / M17^2</f>
@@ -1501,26 +1523,26 @@
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="43"/>
       <c r="C20" s="29" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D20" s="30" t="n">
         <v>0.125</v>
       </c>
       <c r="E20" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F20" s="49" t="n">
         <f aca="false">D20*0.0254</f>
         <v>0.003175</v>
       </c>
       <c r="G20" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H20" s="29"/>
       <c r="I20" s="47"/>
       <c r="K20" s="16"/>
       <c r="L20" s="29" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="M20" s="30" t="n">
         <v>0</v>
@@ -1534,26 +1556,26 @@
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="43"/>
       <c r="C21" s="29" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D21" s="30" t="n">
         <v>36</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F21" s="49" t="n">
         <f aca="false">D21*0.0254</f>
         <v>0.9144</v>
       </c>
       <c r="G21" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H21" s="29"/>
       <c r="I21" s="47"/>
       <c r="K21" s="16"/>
       <c r="L21" s="29" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="M21" s="30" t="n">
         <v>2</v>
@@ -1567,26 +1589,26 @@
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="43"/>
       <c r="C22" s="29" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D22" s="30" t="n">
         <v>1.5</v>
       </c>
       <c r="E22" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F22" s="49" t="n">
         <f aca="false">D22*0.0254</f>
         <v>0.0381</v>
       </c>
       <c r="G22" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H22" s="29"/>
       <c r="I22" s="47"/>
       <c r="K22" s="16"/>
       <c r="L22" s="29" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="M22" s="30" t="n">
         <v>0.5</v>
@@ -1600,26 +1622,26 @@
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="43"/>
       <c r="C23" s="29" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D23" s="30" t="n">
         <v>3</v>
       </c>
       <c r="E23" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F23" s="49" t="n">
         <f aca="false">D23*0.0254</f>
         <v>0.0762</v>
       </c>
       <c r="G23" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H23" s="29"/>
       <c r="I23" s="47"/>
       <c r="K23" s="16"/>
       <c r="L23" s="29" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M23" s="30" t="n">
         <v>0.8</v>
@@ -1633,28 +1655,28 @@
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="43"/>
       <c r="C24" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D24" s="30" t="n">
         <v>22.5</v>
       </c>
       <c r="E24" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F24" s="49" t="n">
         <f aca="false">D24*0.0254</f>
         <v>0.5715</v>
       </c>
       <c r="G24" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H24" s="29" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I24" s="47"/>
       <c r="K24" s="16"/>
       <c r="L24" s="29" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="M24" s="48" t="n">
         <f aca="false">M23*M20+M18 + M22</f>
@@ -1669,26 +1691,26 @@
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="43"/>
       <c r="C25" s="29" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D25" s="50" t="n">
         <f aca="false">F25/0.0254</f>
         <v>0.0393700787401575</v>
       </c>
       <c r="E25" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F25" s="30" t="n">
         <v>0.001</v>
       </c>
       <c r="G25" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H25" s="29"/>
       <c r="I25" s="47"/>
       <c r="K25" s="16"/>
       <c r="L25" s="29" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M25" s="48" t="n">
         <f aca="false">M19 + M23*M21 + M22</f>
@@ -1703,40 +1725,40 @@
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="43"/>
       <c r="C26" s="29" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D26" s="29" t="n">
         <f aca="false">D24+D23-D22</f>
         <v>24</v>
       </c>
       <c r="E26" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F26" s="49" t="n">
         <f aca="false">D26*0.0254</f>
         <v>0.6096</v>
       </c>
       <c r="G26" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H26" s="29"/>
       <c r="I26" s="47"/>
       <c r="K26" s="16"/>
       <c r="L26" s="29" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M26" s="30" t="n">
         <v>15</v>
       </c>
       <c r="N26" s="29" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="O26" s="29" t="n">
         <f aca="false">M26*6895</f>
         <v>103425</v>
       </c>
       <c r="P26" s="29" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q26" s="29"/>
       <c r="R26" s="20"/>
@@ -1744,21 +1766,21 @@
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="43"/>
       <c r="C27" s="29" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D27" s="29" t="n">
         <f aca="false">D21-D22-D24-D23</f>
         <v>9</v>
       </c>
       <c r="E27" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F27" s="49" t="n">
         <f aca="false">D27*0.0254</f>
         <v>0.2286</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H27" s="29"/>
       <c r="I27" s="47"/>
@@ -1792,7 +1814,7 @@
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="43"/>
       <c r="C29" s="44" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D29" s="45"/>
       <c r="E29" s="45"/>
@@ -1812,20 +1834,20 @@
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="43"/>
       <c r="C30" s="29" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D30" s="30" t="n">
         <v>12</v>
       </c>
       <c r="E30" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F30" s="49" t="n">
         <f aca="false">D30*0.0254</f>
         <v>0.3048</v>
       </c>
       <c r="G30" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H30" s="29"/>
       <c r="I30" s="47"/>
@@ -1841,20 +1863,20 @@
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="43"/>
       <c r="C31" s="29" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D31" s="30" t="n">
         <v>0.3125</v>
       </c>
       <c r="E31" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F31" s="49" t="n">
         <f aca="false">D31*0.0254</f>
         <v>0.0079375</v>
       </c>
       <c r="G31" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H31" s="29"/>
       <c r="I31" s="47"/>
@@ -1870,20 +1892,20 @@
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="43"/>
       <c r="C32" s="29" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D32" s="51" t="n">
         <v>3.94E-006</v>
       </c>
       <c r="E32" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F32" s="52" t="n">
         <f aca="false">D32*0.0254</f>
         <v>1.00076E-007</v>
       </c>
       <c r="G32" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H32" s="29"/>
       <c r="I32" s="47"/>
@@ -1899,20 +1921,20 @@
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="43"/>
       <c r="C33" s="29" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D33" s="30" t="n">
         <v>48</v>
       </c>
       <c r="E33" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F33" s="48" t="n">
         <f aca="false">D33*0.0254</f>
         <v>1.2192</v>
       </c>
       <c r="G33" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H33" s="29"/>
       <c r="I33" s="47"/>
@@ -1928,20 +1950,20 @@
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="43"/>
       <c r="C34" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D34" s="30" t="n">
         <v>0.225</v>
       </c>
       <c r="E34" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F34" s="49" t="n">
         <f aca="false">D34*0.0254</f>
         <v>0.005715</v>
       </c>
       <c r="G34" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H34" s="29"/>
       <c r="I34" s="47"/>
@@ -1957,20 +1979,20 @@
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="43"/>
       <c r="C35" s="29" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D35" s="51" t="n">
         <v>3.94E-006</v>
       </c>
       <c r="E35" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F35" s="29" t="n">
         <f aca="false">D35*0.0254</f>
         <v>1.00076E-007</v>
       </c>
       <c r="G35" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H35" s="29"/>
       <c r="I35" s="47"/>
@@ -1996,7 +2018,7 @@
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="43"/>
       <c r="C37" s="44" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D37" s="45"/>
       <c r="E37" s="45"/>
@@ -2008,7 +2030,7 @@
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="43"/>
       <c r="C38" s="29" t="s">
-        <v>72</v>
+        <v>14</v>
       </c>
       <c r="D38" s="30" t="n">
         <v>6</v>
@@ -2022,20 +2044,20 @@
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="43"/>
       <c r="C39" s="29" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D39" s="30" t="n">
         <v>0.089</v>
       </c>
       <c r="E39" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F39" s="49" t="n">
         <f aca="false">D39*0.0254</f>
         <v>0.0022606</v>
       </c>
       <c r="G39" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H39" s="29"/>
       <c r="I39" s="47"/>
@@ -2043,7 +2065,7 @@
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="43"/>
       <c r="C40" s="29" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D40" s="30" t="n">
         <v>0.7</v>
@@ -2057,7 +2079,7 @@
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="43"/>
       <c r="C41" s="29" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="D41" s="30" t="n">
         <v>6</v>
@@ -2077,14 +2099,14 @@
         <v>0.0469</v>
       </c>
       <c r="E42" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F42" s="29" t="n">
         <f aca="false">D42*0.0254</f>
         <v>0.00119126</v>
       </c>
       <c r="G42" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H42" s="29"/>
       <c r="I42" s="47"/>
@@ -2134,14 +2156,14 @@
         <v>2</v>
       </c>
       <c r="E46" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F46" s="49" t="n">
         <f aca="false">D46*0.0254</f>
         <v>0.0508</v>
       </c>
       <c r="G46" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H46" s="29"/>
       <c r="I46" s="47"/>
@@ -2155,14 +2177,14 @@
         <v>0.25</v>
       </c>
       <c r="E47" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F47" s="49" t="n">
         <f aca="false">D47*0.0254</f>
         <v>0.00635</v>
       </c>
       <c r="G47" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H47" s="29"/>
       <c r="I47" s="47"/>
@@ -2176,14 +2198,14 @@
         <v>5</v>
       </c>
       <c r="E48" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F48" s="29" t="n">
         <f aca="false">D48*0.0254</f>
         <v>0.127</v>
       </c>
       <c r="G48" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H48" s="29"/>
       <c r="I48" s="47"/>
@@ -2219,14 +2241,14 @@
         <v>1</v>
       </c>
       <c r="E51" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F51" s="49" t="n">
         <f aca="false">D51*0.0254</f>
         <v>0.0254</v>
       </c>
       <c r="G51" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H51" s="29"/>
       <c r="I51" s="47"/>
@@ -2240,14 +2262,14 @@
         <v>2</v>
       </c>
       <c r="E52" s="29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F52" s="49" t="n">
         <f aca="false">D52*0.0254</f>
         <v>0.0508</v>
       </c>
       <c r="G52" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H52" s="29"/>
       <c r="I52" s="47"/>
@@ -2370,107 +2392,107 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>72</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2515,47 +2537,47 @@
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Results page cleanup; liquid-phase Isp and class percent in title; tank ratio row
- Results page: drop manifold pressures, Isp and c* panels (8 panels now)
- Title shows motor class percent (e.g. K523 (66%)) and average Isp over the
  liquid phase; summary gains average_Isp_liquid and class_percent
- Input sheet: Tank Ratio row, 3 in tank with 0.065 in wall

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="93">
   <si>
     <t xml:space="preserve">Nitrous Tank </t>
   </si>
@@ -104,28 +104,34 @@
     <t xml:space="preserve">Fuel Entrance K-factor</t>
   </si>
   <si>
+    <t xml:space="preserve">Nitrous Ball Valve Cv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Ball Valve Cv</t>
+  </si>
+  <si>
     <t xml:space="preserve">SIMULATION SETUP</t>
   </si>
   <si>
-    <t xml:space="preserve">Nitrous Ball Valve Cv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Ball Valve Cv</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nitrous No. Elbows</t>
   </si>
   <si>
     <t xml:space="preserve">Fuel No. Elbows</t>
   </si>
   <si>
+    <t xml:space="preserve">Nitrous Elbow K-factor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Elbow K-factor</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sweep Setup</t>
   </si>
   <si>
-    <t xml:space="preserve">Nitrous Elbow K-factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Elbow K-factor</t>
+    <t xml:space="preserve">Fuel Piston Loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">psi</t>
   </si>
   <si>
     <t xml:space="preserve">Parameter</t>
@@ -143,15 +149,18 @@
     <t xml:space="preserve">0/1</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuel Piston Loss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">psi</t>
+    <t xml:space="preserve">grid size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exit Diameter</t>
   </si>
   <si>
     <t xml:space="preserve">Tank</t>
   </si>
   <si>
+    <t xml:space="preserve">Tank OD</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ambient Conditions</t>
   </si>
   <si>
@@ -161,7 +170,7 @@
     <t xml:space="preserve">metric</t>
   </si>
   <si>
-    <t xml:space="preserve">Tank OD</t>
+    <t xml:space="preserve">Tank Wall Thickness</t>
   </si>
   <si>
     <t xml:space="preserve">Timestep</t>
@@ -170,13 +179,13 @@
     <t xml:space="preserve">s</t>
   </si>
   <si>
-    <t xml:space="preserve">Tank Wall Thickness</t>
+    <t xml:space="preserve">Bulkhead Insertion Length</t>
   </si>
   <si>
     <t xml:space="preserve">Sim Max Duration</t>
   </si>
   <si>
-    <t xml:space="preserve">Bulkhead Insertion Length</t>
+    <t xml:space="preserve">Piston Length</t>
   </si>
   <si>
     <t xml:space="preserve">Nitrous Temperature</t>
@@ -191,7 +200,7 @@
     <t xml:space="preserve">10 F less than ambient</t>
   </si>
   <si>
-    <t xml:space="preserve">Piston Length</t>
+    <t xml:space="preserve">Static Vent Diameter</t>
   </si>
   <si>
     <t xml:space="preserve">Ambient Pressure</t>
@@ -203,12 +212,15 @@
     <t xml:space="preserve">Ambient at FAR</t>
   </si>
   <si>
-    <t xml:space="preserve">Static Vent Diameter</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tank Length</t>
   </si>
   <si>
+    <t xml:space="preserve">Tank Ratio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vox/Vfuel, 2.15</t>
+  </si>
+  <si>
     <t xml:space="preserve">Propellant Properties</t>
   </si>
   <si>
@@ -224,6 +236,9 @@
     <t xml:space="preserve">Isopropanol</t>
   </si>
   <si>
+    <t xml:space="preserve">             </t>
+  </si>
+  <si>
     <t xml:space="preserve">Fuel Density</t>
   </si>
   <si>
@@ -233,9 +248,6 @@
     <t xml:space="preserve">Chamber </t>
   </si>
   <si>
-    <t xml:space="preserve">             </t>
-  </si>
-  <si>
     <t xml:space="preserve">Fuel Dynamic Viscosity</t>
   </si>
   <si>
@@ -273,9 +285,6 @@
   </si>
   <si>
     <t xml:space="preserve">Decay Constant (liquid)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exit Diameter</t>
   </si>
   <si>
     <t xml:space="preserve">Decay Constant (vapor)</t>
@@ -297,12 +306,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.00E+00"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="0.00"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -509,7 +519,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -687,6 +697,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -698,15 +720,15 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -718,15 +740,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -734,11 +748,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -750,10 +764,6 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -763,6 +773,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1245,7 +1259,7 @@
         <v>3</v>
       </c>
       <c r="M5" s="27" t="n">
-        <v>22.5</v>
+        <v>14.25</v>
       </c>
       <c r="N5" s="27" t="s">
         <v>4</v>
@@ -1258,7 +1272,7 @@
         <v>5</v>
       </c>
       <c r="T5" s="27" t="n">
-        <v>10.5</v>
+        <v>6.75</v>
       </c>
       <c r="U5" s="27" t="s">
         <v>4</v>
@@ -1360,7 +1374,7 @@
         <v>8</v>
       </c>
       <c r="M8" s="27" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="N8" s="27"/>
       <c r="O8" s="27"/>
@@ -1401,7 +1415,7 @@
         <v>10</v>
       </c>
       <c r="M9" s="27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N9" s="27"/>
       <c r="O9" s="27"/>
@@ -1412,7 +1426,7 @@
         <v>11</v>
       </c>
       <c r="T9" s="27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U9" s="27"/>
       <c r="V9" s="27"/>
@@ -1488,7 +1502,7 @@
       </c>
       <c r="M11" s="30" t="n">
         <f aca="false">PI()/4*M10^2*M9</f>
-        <v>0.0373268331136271</v>
+        <v>0.0248845554090847</v>
       </c>
       <c r="N11" s="29" t="s">
         <v>15</v>
@@ -1502,7 +1516,7 @@
       </c>
       <c r="T11" s="30" t="n">
         <f aca="false">PI()/4*T10^2*T9</f>
-        <v>0.0117809724509617</v>
+        <v>0.00785398163397448</v>
       </c>
       <c r="U11" s="29" t="s">
         <v>15</v>
@@ -1617,7 +1631,7 @@
         <v>20</v>
       </c>
       <c r="T14" s="27" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="U14" s="27" t="s">
         <v>4</v>
@@ -1726,14 +1740,14 @@
       <c r="AG16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="34"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="35"/>
-      <c r="I17" s="36"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="16"/>
       <c r="K17" s="17"/>
       <c r="L17" s="27" t="s">
         <v>25</v>
@@ -1767,12 +1781,17 @@
       <c r="AG17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="37" t="s">
-        <v>27</v>
-      </c>
+      <c r="B18" s="34"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
+      <c r="G18" s="35"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="36"/>
       <c r="K18" s="17"/>
       <c r="L18" s="27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M18" s="27" t="n">
         <v>1.6</v>
@@ -1783,7 +1802,7 @@
       <c r="Q18" s="3"/>
       <c r="R18" s="22"/>
       <c r="S18" s="27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="T18" s="27" t="n">
         <v>1.6</v>
@@ -1803,14 +1822,9 @@
       <c r="AG18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="38"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="39"/>
-      <c r="I19" s="40"/>
+      <c r="B19" s="37" t="s">
+        <v>29</v>
+      </c>
       <c r="K19" s="17"/>
       <c r="L19" s="27" t="s">
         <v>30</v>
@@ -1844,19 +1858,17 @@
       <c r="AG19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="41"/>
-      <c r="C20" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="43"/>
-      <c r="E20" s="43"/>
-      <c r="F20" s="43"/>
-      <c r="G20" s="43"/>
-      <c r="H20" s="43"/>
-      <c r="I20" s="44"/>
+      <c r="B20" s="38"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="39"/>
+      <c r="I20" s="40"/>
       <c r="K20" s="17"/>
       <c r="L20" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M20" s="27" t="n">
         <v>0.8</v>
@@ -1867,7 +1879,7 @@
       <c r="Q20" s="3"/>
       <c r="R20" s="22"/>
       <c r="S20" s="27" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="T20" s="27" t="n">
         <v>0.8</v>
@@ -1888,38 +1900,30 @@
     </row>
     <row r="21" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="41"/>
-      <c r="C21" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="D21" s="45" t="s">
-        <v>36</v>
-      </c>
-      <c r="E21" s="46" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="G21" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="H21" s="27"/>
+      <c r="C21" s="42" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="43"/>
       <c r="I21" s="44"/>
-      <c r="K21" s="47"/>
-      <c r="L21" s="48"/>
-      <c r="M21" s="48"/>
-      <c r="N21" s="48"/>
-      <c r="O21" s="48"/>
-      <c r="P21" s="49"/>
+      <c r="K21" s="45"/>
+      <c r="L21" s="46"/>
+      <c r="M21" s="46"/>
+      <c r="N21" s="46"/>
+      <c r="O21" s="46"/>
+      <c r="P21" s="47"/>
       <c r="R21" s="22"/>
       <c r="S21" s="27" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="T21" s="27" t="n">
         <v>15</v>
       </c>
       <c r="U21" s="27" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="V21" s="27"/>
       <c r="W21" s="26"/>
@@ -1937,31 +1941,30 @@
     <row r="22" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="41"/>
       <c r="C22" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="D22" s="50" t="n">
-        <v>6</v>
-      </c>
-      <c r="E22" s="51" t="n">
-        <v>36</v>
-      </c>
-      <c r="F22" s="50" t="n">
-        <v>6</v>
-      </c>
-      <c r="G22" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="27" t="n">
-        <f aca="false">(E22-D22)/F22 + 1</f>
-        <v>6</v>
+        <v>37</v>
+      </c>
+      <c r="D22" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="49" t="s">
+        <v>39</v>
+      </c>
+      <c r="F22" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="G22" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="H22" s="27" t="s">
+        <v>42</v>
       </c>
       <c r="I22" s="44"/>
-      <c r="R22" s="52"/>
-      <c r="S22" s="53"/>
-      <c r="T22" s="53"/>
-      <c r="U22" s="53"/>
-      <c r="V22" s="53"/>
-      <c r="W22" s="54"/>
+      <c r="R22" s="50"/>
+      <c r="S22" s="51"/>
+      <c r="T22" s="51"/>
+      <c r="U22" s="51"/>
+      <c r="V22" s="51"/>
+      <c r="W22" s="52"/>
       <c r="X22" s="3"/>
       <c r="Y22" s="4"/>
       <c r="Z22" s="2"/>
@@ -1976,23 +1979,23 @@
     <row r="23" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="41"/>
       <c r="C23" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" s="50" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E23" s="51" t="n">
+        <v>43</v>
+      </c>
+      <c r="D23" s="53" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E23" s="54" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="F23" s="53" t="n">
         <v>0.1</v>
       </c>
-      <c r="F23" s="50" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="G23" s="51" t="n">
+      <c r="G23" s="54" t="n">
         <v>0</v>
       </c>
       <c r="H23" s="27" t="n">
         <f aca="false">(E23-D23)/F23 + 1</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I23" s="44"/>
       <c r="K23" s="38"/>
@@ -2008,19 +2011,32 @@
     </row>
     <row r="24" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="41"/>
-      <c r="C24" s="55"/>
-      <c r="D24" s="55"/>
-      <c r="E24" s="55"/>
-      <c r="F24" s="55"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="55"/>
+      <c r="C24" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="53" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E24" s="54" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F24" s="53" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="G24" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="27" t="n">
+        <f aca="false">(E24-D24)/F24 + 1</f>
+        <v>5</v>
+      </c>
       <c r="I24" s="44"/>
       <c r="K24" s="41"/>
-      <c r="L24" s="56" t="s">
-        <v>42</v>
-      </c>
-      <c r="M24" s="55"/>
-      <c r="N24" s="55"/>
+      <c r="L24" s="55" t="s">
+        <v>44</v>
+      </c>
+      <c r="M24" s="56"/>
+      <c r="N24" s="56"/>
       <c r="O24" s="57" t="s">
         <v>1</v>
       </c>
@@ -2032,33 +2048,25 @@
     </row>
     <row r="25" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="41"/>
-      <c r="C25" s="56" t="s">
-        <v>43</v>
-      </c>
-      <c r="D25" s="58" t="s">
-        <v>44</v>
-      </c>
-      <c r="E25" s="58"/>
-      <c r="F25" s="58" t="s">
-        <v>45</v>
-      </c>
-      <c r="G25" s="58"/>
-      <c r="H25" s="59" t="s">
-        <v>1</v>
-      </c>
+      <c r="C25" s="56"/>
+      <c r="D25" s="56"/>
+      <c r="E25" s="56"/>
+      <c r="F25" s="56"/>
+      <c r="G25" s="56"/>
+      <c r="H25" s="56"/>
       <c r="I25" s="44"/>
       <c r="K25" s="41"/>
       <c r="L25" s="27" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M25" s="27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N25" s="27" t="s">
         <v>4</v>
       </c>
       <c r="O25" s="27"/>
-      <c r="P25" s="60"/>
+      <c r="P25" s="58"/>
       <c r="Q25" s="3"/>
       <c r="X25" s="3"/>
       <c r="Y25" s="4"/>
@@ -2067,31 +2075,33 @@
     </row>
     <row r="26" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="41"/>
-      <c r="C26" s="27" t="s">
+      <c r="C26" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="D26" s="27" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E26" s="27" t="s">
+      <c r="E26" s="59"/>
+      <c r="F26" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="F26" s="27"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="27"/>
+      <c r="G26" s="59"/>
+      <c r="H26" s="60" t="s">
+        <v>1</v>
+      </c>
       <c r="I26" s="44"/>
       <c r="K26" s="41"/>
       <c r="L26" s="27" t="s">
         <v>49</v>
       </c>
       <c r="M26" s="27" t="n">
-        <v>0.125</v>
+        <v>0.065</v>
       </c>
       <c r="N26" s="27" t="s">
         <v>4</v>
       </c>
       <c r="O26" s="27"/>
-      <c r="P26" s="60"/>
+      <c r="P26" s="58"/>
       <c r="Q26" s="4"/>
       <c r="X26" s="3"/>
       <c r="Y26" s="4"/>
@@ -2104,10 +2114,10 @@
         <v>50</v>
       </c>
       <c r="D27" s="27" t="n">
-        <v>30</v>
+        <v>0.01</v>
       </c>
       <c r="E27" s="27" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F27" s="27"/>
       <c r="G27" s="27"/>
@@ -2115,7 +2125,7 @@
       <c r="I27" s="44"/>
       <c r="K27" s="41"/>
       <c r="L27" s="27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M27" s="27" t="n">
         <v>1.5</v>
@@ -2124,7 +2134,7 @@
         <v>4</v>
       </c>
       <c r="O27" s="27"/>
-      <c r="P27" s="60"/>
+      <c r="P27" s="58"/>
       <c r="Q27" s="61"/>
       <c r="X27" s="3"/>
       <c r="Y27" s="4"/>
@@ -2134,28 +2144,21 @@
     <row r="28" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="41"/>
       <c r="C28" s="27" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="E28" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="F28" s="62" t="n">
-        <f aca="false">(D28-32)/1.8</f>
-        <v>10</v>
-      </c>
-      <c r="G28" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="H28" s="27" t="s">
-        <v>55</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="27"/>
       <c r="I28" s="44"/>
       <c r="K28" s="41"/>
       <c r="L28" s="27" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="M28" s="27" t="n">
         <v>3</v>
@@ -2164,7 +2167,7 @@
         <v>4</v>
       </c>
       <c r="O28" s="27"/>
-      <c r="P28" s="60"/>
+      <c r="P28" s="58"/>
       <c r="Q28" s="61"/>
       <c r="X28" s="3"/>
       <c r="Y28" s="4"/>
@@ -2174,28 +2177,28 @@
     <row r="29" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="41"/>
       <c r="C29" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="D29" s="27" t="n">
+        <v>50</v>
+      </c>
+      <c r="E29" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="F29" s="62" t="n">
+        <f aca="false">(D29-32)/1.8</f>
+        <v>10</v>
+      </c>
+      <c r="G29" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="D29" s="27" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="E29" s="27" t="s">
-        <v>41</v>
-      </c>
-      <c r="F29" s="27" t="n">
-        <f aca="false">D29*6895</f>
-        <v>93082.5</v>
-      </c>
-      <c r="G29" s="27" t="s">
+      <c r="H29" s="27" t="s">
         <v>58</v>
-      </c>
-      <c r="H29" s="27" t="s">
-        <v>59</v>
       </c>
       <c r="I29" s="44"/>
       <c r="K29" s="41"/>
       <c r="L29" s="27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M29" s="27" t="n">
         <v>0.04</v>
@@ -2204,7 +2207,7 @@
         <v>4</v>
       </c>
       <c r="O29" s="27"/>
-      <c r="P29" s="60"/>
+      <c r="P29" s="58"/>
       <c r="Q29" s="61"/>
       <c r="X29" s="3"/>
       <c r="Y29" s="4"/>
@@ -2213,20 +2216,33 @@
     </row>
     <row r="30" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="41"/>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="55"/>
-      <c r="G30" s="55"/>
-      <c r="H30" s="55"/>
+      <c r="C30" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="27" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E30" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="F30" s="27" t="n">
+        <f aca="false">D30*6895</f>
+        <v>93082.5</v>
+      </c>
+      <c r="G30" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="H30" s="27" t="s">
+        <v>62</v>
+      </c>
       <c r="I30" s="44"/>
       <c r="K30" s="41"/>
       <c r="L30" s="27" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="M30" s="63" t="n">
         <f aca="false">2*M27 + M5+T5</f>
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="N30" s="27" t="s">
         <v>4</v>
@@ -2241,28 +2257,24 @@
     </row>
     <row r="31" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="41"/>
-      <c r="C31" s="42" t="s">
-        <v>62</v>
-      </c>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="43"/>
-      <c r="H31" s="43"/>
+      <c r="C31" s="56"/>
+      <c r="D31" s="56"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="56"/>
+      <c r="G31" s="56"/>
+      <c r="H31" s="56"/>
       <c r="I31" s="44"/>
       <c r="K31" s="41"/>
       <c r="L31" s="27" t="s">
-        <v>63</v>
-      </c>
-      <c r="M31" s="63" t="n">
-        <f aca="false">M27+M5-M28</f>
-        <v>21</v>
-      </c>
-      <c r="N31" s="27" t="s">
-        <v>4</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="M31" s="64" t="n">
+        <f aca="false">M5/T5</f>
+        <v>2.11111111111111</v>
+      </c>
+      <c r="N31" s="27"/>
       <c r="O31" s="27" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P31" s="44"/>
       <c r="Q31" s="61"/>
@@ -2273,22 +2285,29 @@
     </row>
     <row r="32" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="41"/>
-      <c r="C32" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" s="64" t="s">
+      <c r="C32" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="E32" s="64"/>
-      <c r="F32" s="65"/>
-      <c r="G32" s="65"/>
-      <c r="H32" s="65"/>
+      <c r="D32" s="43"/>
+      <c r="E32" s="43"/>
+      <c r="F32" s="43"/>
+      <c r="G32" s="43"/>
+      <c r="H32" s="43"/>
       <c r="I32" s="44"/>
       <c r="K32" s="41"/>
-      <c r="L32" s="55"/>
-      <c r="M32" s="55"/>
-      <c r="N32" s="55"/>
-      <c r="O32" s="55"/>
+      <c r="L32" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="M32" s="63" t="n">
+        <f aca="false">M27+M5-M28</f>
+        <v>12.75</v>
+      </c>
+      <c r="N32" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="O32" s="27" t="s">
+        <v>68</v>
+      </c>
       <c r="P32" s="44"/>
       <c r="Q32" s="3"/>
       <c r="X32" s="3"/>
@@ -2299,29 +2318,25 @@
     <row r="33" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="41"/>
       <c r="C33" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27" t="n">
-        <v>786</v>
-      </c>
-      <c r="G33" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="H33" s="27"/>
+        <v>69</v>
+      </c>
+      <c r="D33" s="65" t="s">
+        <v>70</v>
+      </c>
+      <c r="E33" s="65"/>
+      <c r="F33" s="66"/>
+      <c r="G33" s="66"/>
+      <c r="H33" s="66"/>
       <c r="I33" s="44"/>
       <c r="K33" s="41"/>
-      <c r="L33" s="56" t="s">
-        <v>69</v>
-      </c>
-      <c r="M33" s="55"/>
-      <c r="N33" s="55"/>
-      <c r="O33" s="55"/>
+      <c r="L33" s="56"/>
+      <c r="M33" s="56"/>
+      <c r="N33" s="56"/>
+      <c r="O33" s="56"/>
       <c r="P33" s="44"/>
       <c r="Q33" s="3"/>
       <c r="T33" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Y33" s="2"/>
       <c r="AF33" s="2"/>
@@ -2330,29 +2345,25 @@
     <row r="34" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="41"/>
       <c r="C34" s="27" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D34" s="27"/>
       <c r="E34" s="27"/>
       <c r="F34" s="27" t="n">
-        <v>2.5</v>
+        <v>786</v>
       </c>
       <c r="G34" s="27" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H34" s="27"/>
       <c r="I34" s="44"/>
-      <c r="K34" s="66"/>
-      <c r="L34" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="M34" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="N34" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="O34" s="27"/>
+      <c r="K34" s="41"/>
+      <c r="L34" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="M34" s="56"/>
+      <c r="N34" s="56"/>
+      <c r="O34" s="56"/>
       <c r="P34" s="44"/>
       <c r="Q34" s="3"/>
       <c r="Y34" s="2"/>
@@ -2362,26 +2373,24 @@
     <row r="35" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="41"/>
       <c r="C35" s="27" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D35" s="27"/>
       <c r="E35" s="27"/>
       <c r="F35" s="27" t="n">
-        <v>0.07</v>
+        <v>2.5</v>
       </c>
       <c r="G35" s="27" t="s">
-        <v>72</v>
-      </c>
-      <c r="H35" s="27" t="s">
-        <v>75</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="H35" s="27"/>
       <c r="I35" s="44"/>
-      <c r="K35" s="66"/>
+      <c r="K35" s="67"/>
       <c r="L35" s="27" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M35" s="27" t="n">
-        <v>0.25</v>
+        <v>1.5</v>
       </c>
       <c r="N35" s="27" t="s">
         <v>4</v>
@@ -2395,19 +2404,27 @@
     </row>
     <row r="36" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="41"/>
-      <c r="C36" s="43"/>
-      <c r="D36" s="43"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="43"/>
+      <c r="C36" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
+      <c r="F36" s="27" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="G36" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="H36" s="27" t="s">
+        <v>79</v>
+      </c>
       <c r="I36" s="44"/>
-      <c r="K36" s="66"/>
+      <c r="K36" s="67"/>
       <c r="L36" s="27" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="M36" s="27" t="n">
-        <v>5</v>
+        <v>0.25</v>
       </c>
       <c r="N36" s="27" t="s">
         <v>4</v>
@@ -2420,20 +2437,24 @@
     </row>
     <row r="37" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="41"/>
-      <c r="C37" s="56" t="s">
-        <v>78</v>
-      </c>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="55"/>
-      <c r="G37" s="55"/>
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
+      <c r="F37" s="43"/>
+      <c r="G37" s="43"/>
       <c r="H37" s="43"/>
       <c r="I37" s="44"/>
-      <c r="K37" s="66"/>
-      <c r="L37" s="43"/>
-      <c r="M37" s="43"/>
-      <c r="N37" s="43"/>
-      <c r="O37" s="43"/>
+      <c r="K37" s="67"/>
+      <c r="L37" s="27" t="s">
+        <v>81</v>
+      </c>
+      <c r="M37" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="N37" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="O37" s="27"/>
       <c r="P37" s="44"/>
       <c r="Y37" s="2"/>
       <c r="AF37" s="2"/>
@@ -2441,59 +2462,51 @@
     </row>
     <row r="38" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="41"/>
-      <c r="C38" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D38" s="27" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="E38" s="27"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
+      <c r="C38" s="55" t="s">
+        <v>82</v>
+      </c>
+      <c r="D38" s="56"/>
+      <c r="E38" s="56"/>
+      <c r="F38" s="56"/>
+      <c r="G38" s="56"/>
+      <c r="H38" s="43"/>
       <c r="I38" s="44"/>
-      <c r="K38" s="66"/>
-      <c r="L38" s="56" t="s">
-        <v>80</v>
-      </c>
-      <c r="M38" s="55"/>
-      <c r="N38" s="55"/>
-      <c r="O38" s="55"/>
+      <c r="K38" s="67"/>
+      <c r="L38" s="43"/>
+      <c r="M38" s="43"/>
+      <c r="N38" s="43"/>
+      <c r="O38" s="43"/>
       <c r="P38" s="44"/>
     </row>
     <row r="39" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="41"/>
       <c r="C39" s="27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D39" s="27" t="n">
-        <v>0.95</v>
+        <v>0.65</v>
       </c>
       <c r="E39" s="27"/>
       <c r="F39" s="27"/>
       <c r="G39" s="27"/>
       <c r="H39" s="27"/>
       <c r="I39" s="44"/>
-      <c r="K39" s="41"/>
-      <c r="L39" s="27" t="s">
-        <v>82</v>
-      </c>
-      <c r="M39" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="N39" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="O39" s="27"/>
+      <c r="K39" s="67"/>
+      <c r="L39" s="55" t="s">
+        <v>84</v>
+      </c>
+      <c r="M39" s="56"/>
+      <c r="N39" s="56"/>
+      <c r="O39" s="56"/>
       <c r="P39" s="44"/>
     </row>
     <row r="40" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="41"/>
       <c r="C40" s="27" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>0.7</v>
+        <v>0.95</v>
       </c>
       <c r="E40" s="27"/>
       <c r="F40" s="27"/>
@@ -2502,10 +2515,10 @@
       <c r="I40" s="44"/>
       <c r="K40" s="41"/>
       <c r="L40" s="27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="M40" s="27" t="n">
-        <v>1.7</v>
+        <v>0.75</v>
       </c>
       <c r="N40" s="27" t="s">
         <v>4</v>
@@ -2516,70 +2529,99 @@
     <row r="41" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="41"/>
       <c r="C41" s="27" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D41" s="27" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E41" s="27" t="s">
-        <v>86</v>
-      </c>
+        <v>0.7</v>
+      </c>
+      <c r="E41" s="27"/>
       <c r="F41" s="27"/>
       <c r="G41" s="27"/>
       <c r="H41" s="27"/>
       <c r="I41" s="44"/>
       <c r="K41" s="41"/>
       <c r="L41" s="27" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="M41" s="27" t="n">
-        <v>15</v>
+        <v>1.25</v>
       </c>
       <c r="N41" s="27" t="s">
-        <v>88</v>
+        <v>4</v>
       </c>
       <c r="O41" s="27"/>
       <c r="P41" s="44"/>
     </row>
     <row r="42" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="67"/>
-      <c r="C42" s="68"/>
-      <c r="D42" s="68"/>
-      <c r="E42" s="68"/>
-      <c r="F42" s="68"/>
-      <c r="G42" s="68"/>
-      <c r="H42" s="68"/>
-      <c r="I42" s="69"/>
-      <c r="K42" s="67"/>
-      <c r="L42" s="68"/>
-      <c r="M42" s="68"/>
-      <c r="N42" s="68"/>
-      <c r="O42" s="68"/>
-      <c r="P42" s="69"/>
+      <c r="B42" s="41"/>
+      <c r="C42" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="D42" s="27" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E42" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="F42" s="27"/>
+      <c r="G42" s="27"/>
+      <c r="H42" s="27"/>
+      <c r="I42" s="44"/>
+      <c r="K42" s="41"/>
+      <c r="L42" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="M42" s="27" t="n">
+        <v>15</v>
+      </c>
+      <c r="N42" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="O42" s="27"/>
+      <c r="P42" s="44"/>
+    </row>
+    <row r="43" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B43" s="68"/>
+      <c r="C43" s="69"/>
+      <c r="D43" s="69"/>
+      <c r="E43" s="69"/>
+      <c r="F43" s="69"/>
+      <c r="G43" s="69"/>
+      <c r="H43" s="69"/>
+      <c r="I43" s="70"/>
+      <c r="K43" s="68"/>
+      <c r="L43" s="69"/>
+      <c r="M43" s="69"/>
+      <c r="N43" s="69"/>
+      <c r="O43" s="69"/>
+      <c r="P43" s="70"/>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:H33"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D32" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D33" type="list">
       <formula1>"Isopropanol,Ethanol,E98,E85"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C24" type="none"/>
-    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G22:G23" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C25" type="none">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G23:G24" type="list">
       <formula1>"0,1"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="F22:F23" type="none">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="F23:F24" type="none">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C22:C23" type="list">
+    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C23:C24" type="list">
       <formula1>lists!$A$2:$A$43</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2607,62 +2649,62 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2707,7 +2749,7 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2717,12 +2759,12 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2732,32 +2774,32 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>84</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2802,7 +2844,7 @@
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2812,12 +2854,12 @@
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Input sheet: 2D sweep of exit x throat diameter; exit diameter 1.2 in
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -155,6 +155,9 @@
     <t xml:space="preserve">Exit Diameter</t>
   </si>
   <si>
+    <t xml:space="preserve">Throat Diameter</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tank</t>
   </si>
   <si>
@@ -279,9 +282,6 @@
   </si>
   <si>
     <t xml:space="preserve">Nozzle Efficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Throat Diameter</t>
   </si>
   <si>
     <t xml:space="preserve">Decay Constant (liquid)</t>
@@ -1982,20 +1982,20 @@
         <v>43</v>
       </c>
       <c r="D23" s="53" t="n">
-        <v>1.05</v>
+        <v>1</v>
       </c>
       <c r="E23" s="54" t="n">
-        <v>1.65</v>
+        <v>1.5</v>
       </c>
       <c r="F23" s="53" t="n">
         <v>0.1</v>
       </c>
       <c r="G23" s="54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23" s="27" t="n">
         <f aca="false">(E23-D23)/F23 + 1</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I23" s="44"/>
       <c r="K23" s="38"/>
@@ -2012,28 +2012,28 @@
     <row r="24" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="41"/>
       <c r="C24" s="27" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="D24" s="53" t="n">
-        <v>0.08</v>
+        <v>0.6</v>
       </c>
       <c r="E24" s="54" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F24" s="53" t="n">
         <v>0.1</v>
       </c>
-      <c r="F24" s="53" t="n">
-        <v>0.005</v>
-      </c>
       <c r="G24" s="54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" s="27" t="n">
         <f aca="false">(E24-D24)/F24 + 1</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I24" s="44"/>
       <c r="K24" s="41"/>
       <c r="L24" s="55" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M24" s="56"/>
       <c r="N24" s="56"/>
@@ -2057,7 +2057,7 @@
       <c r="I25" s="44"/>
       <c r="K25" s="41"/>
       <c r="L25" s="27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M25" s="27" t="n">
         <v>3</v>
@@ -2076,14 +2076,14 @@
     <row r="26" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="41"/>
       <c r="C26" s="55" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D26" s="59" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E26" s="59"/>
       <c r="F26" s="59" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G26" s="59"/>
       <c r="H26" s="60" t="s">
@@ -2092,7 +2092,7 @@
       <c r="I26" s="44"/>
       <c r="K26" s="41"/>
       <c r="L26" s="27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M26" s="27" t="n">
         <v>0.065</v>
@@ -2111,13 +2111,13 @@
     <row r="27" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="41"/>
       <c r="C27" s="27" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D27" s="27" t="n">
         <v>0.01</v>
       </c>
       <c r="E27" s="27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F27" s="27"/>
       <c r="G27" s="27"/>
@@ -2125,7 +2125,7 @@
       <c r="I27" s="44"/>
       <c r="K27" s="41"/>
       <c r="L27" s="27" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M27" s="27" t="n">
         <v>1.5</v>
@@ -2144,13 +2144,13 @@
     <row r="28" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="41"/>
       <c r="C28" s="27" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D28" s="27" t="n">
         <v>30</v>
       </c>
       <c r="E28" s="27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F28" s="27"/>
       <c r="G28" s="27"/>
@@ -2158,7 +2158,7 @@
       <c r="I28" s="44"/>
       <c r="K28" s="41"/>
       <c r="L28" s="27" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M28" s="27" t="n">
         <v>3</v>
@@ -2177,28 +2177,28 @@
     <row r="29" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="41"/>
       <c r="C29" s="27" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D29" s="27" t="n">
         <v>50</v>
       </c>
       <c r="E29" s="27" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F29" s="62" t="n">
         <f aca="false">(D29-32)/1.8</f>
         <v>10</v>
       </c>
       <c r="G29" s="27" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H29" s="27" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I29" s="44"/>
       <c r="K29" s="41"/>
       <c r="L29" s="27" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="M29" s="27" t="n">
         <v>0.04</v>
@@ -2217,7 +2217,7 @@
     <row r="30" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="41"/>
       <c r="C30" s="27" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D30" s="27" t="n">
         <v>13.5</v>
@@ -2230,15 +2230,15 @@
         <v>93082.5</v>
       </c>
       <c r="G30" s="27" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H30" s="27" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I30" s="44"/>
       <c r="K30" s="41"/>
       <c r="L30" s="27" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M30" s="63" t="n">
         <f aca="false">2*M27 + M5+T5</f>
@@ -2266,7 +2266,7 @@
       <c r="I31" s="44"/>
       <c r="K31" s="41"/>
       <c r="L31" s="27" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="M31" s="64" t="n">
         <f aca="false">M5/T5</f>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="N31" s="27"/>
       <c r="O31" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P31" s="44"/>
       <c r="Q31" s="61"/>
@@ -2286,7 +2286,7 @@
     <row r="32" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="41"/>
       <c r="C32" s="42" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D32" s="43"/>
       <c r="E32" s="43"/>
@@ -2296,7 +2296,7 @@
       <c r="I32" s="44"/>
       <c r="K32" s="41"/>
       <c r="L32" s="27" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M32" s="63" t="n">
         <f aca="false">M27+M5-M28</f>
@@ -2306,7 +2306,7 @@
         <v>4</v>
       </c>
       <c r="O32" s="27" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="P32" s="44"/>
       <c r="Q32" s="3"/>
@@ -2318,10 +2318,10 @@
     <row r="33" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="41"/>
       <c r="C33" s="27" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D33" s="65" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E33" s="65"/>
       <c r="F33" s="66"/>
@@ -2336,7 +2336,7 @@
       <c r="P33" s="44"/>
       <c r="Q33" s="3"/>
       <c r="T33" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Y33" s="2"/>
       <c r="AF33" s="2"/>
@@ -2345,7 +2345,7 @@
     <row r="34" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="41"/>
       <c r="C34" s="27" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D34" s="27"/>
       <c r="E34" s="27"/>
@@ -2353,13 +2353,13 @@
         <v>786</v>
       </c>
       <c r="G34" s="27" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H34" s="27"/>
       <c r="I34" s="44"/>
       <c r="K34" s="41"/>
       <c r="L34" s="55" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M34" s="56"/>
       <c r="N34" s="56"/>
@@ -2373,7 +2373,7 @@
     <row r="35" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="41"/>
       <c r="C35" s="27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D35" s="27"/>
       <c r="E35" s="27"/>
@@ -2381,13 +2381,13 @@
         <v>2.5</v>
       </c>
       <c r="G35" s="27" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H35" s="27"/>
       <c r="I35" s="44"/>
       <c r="K35" s="67"/>
       <c r="L35" s="27" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M35" s="27" t="n">
         <v>1.5</v>
@@ -2405,7 +2405,7 @@
     <row r="36" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="41"/>
       <c r="C36" s="27" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D36" s="27"/>
       <c r="E36" s="27"/>
@@ -2413,15 +2413,15 @@
         <v>0.07</v>
       </c>
       <c r="G36" s="27" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H36" s="27" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I36" s="44"/>
       <c r="K36" s="67"/>
       <c r="L36" s="27" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="M36" s="27" t="n">
         <v>0.25</v>
@@ -2446,7 +2446,7 @@
       <c r="I37" s="44"/>
       <c r="K37" s="67"/>
       <c r="L37" s="27" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M37" s="27" t="n">
         <v>4</v>
@@ -2463,7 +2463,7 @@
     <row r="38" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="41"/>
       <c r="C38" s="55" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D38" s="56"/>
       <c r="E38" s="56"/>
@@ -2481,7 +2481,7 @@
     <row r="39" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="41"/>
       <c r="C39" s="27" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D39" s="27" t="n">
         <v>0.65</v>
@@ -2493,7 +2493,7 @@
       <c r="I39" s="44"/>
       <c r="K39" s="67"/>
       <c r="L39" s="55" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M39" s="56"/>
       <c r="N39" s="56"/>
@@ -2503,7 +2503,7 @@
     <row r="40" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="41"/>
       <c r="C40" s="27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D40" s="27" t="n">
         <v>0.95</v>
@@ -2515,7 +2515,7 @@
       <c r="I40" s="44"/>
       <c r="K40" s="41"/>
       <c r="L40" s="27" t="s">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="M40" s="27" t="n">
         <v>0.75</v>
@@ -2544,7 +2544,7 @@
         <v>43</v>
       </c>
       <c r="M41" s="27" t="n">
-        <v>1.25</v>
+        <v>1.2</v>
       </c>
       <c r="N41" s="27" t="s">
         <v>4</v>
@@ -2654,47 +2654,47 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2764,32 +2764,32 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>86</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Drill size dropdowns for nitrous and fuel hole diameters
Hole diameters are picked from standard US drill sizes (#80-#39 and 1/64-3/32 in,
up to 0.1 in) on the input sheet; the diameter cells look the size up from a drill
table on the lists sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="143">
   <si>
     <t xml:space="preserve">Nitrous Tank </t>
   </si>
@@ -62,9 +62,15 @@
     <t xml:space="preserve">Nitrous Hole Diameter</t>
   </si>
   <si>
+    <t xml:space="preserve">#54 (0.0550)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fuel Hole Diameter</t>
   </si>
   <si>
+    <t xml:space="preserve">1/32 (0.0312)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nitrous Injector Area</t>
   </si>
   <si>
@@ -300,6 +306,150 @@
   </si>
   <si>
     <t xml:space="preserve">Sweepable parameters (dropdown source for the sweep block)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drill sizes (dropdown source for hole diameters)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diameter [in]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#80 (0.0135)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#79 (0.0145)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/64 (0.0156)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#78 (0.0160)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#77 (0.0180)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#76 (0.0200)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#75 (0.0210)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#74 (0.0225)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#73 (0.0240)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#72 (0.0250)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#71 (0.0260)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#70 (0.0280)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#69 (0.0292)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#68 (0.0310)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#67 (0.0320)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#66 (0.0330)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#65 (0.0350)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#64 (0.0360)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#63 (0.0370)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#62 (0.0380)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#61 (0.0390)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#60 (0.0400)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#59 (0.0410)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#58 (0.0420)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#57 (0.0430)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#56 (0.0465)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/64 (0.0469)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#55 (0.0520)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#53 (0.0595)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/16 (0.0625)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#52 (0.0635)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#51 (0.0670)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#50 (0.0700)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#49 (0.0730)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#48 (0.0760)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5/64 (0.0781)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#47 (0.0785)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#46 (0.0810)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#45 (0.0820)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#44 (0.0860)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#43 (0.0890)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#42 (0.0935)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/32 (0.0938)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#41 (0.0960)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#40 (0.0980)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#39 (0.0995)</t>
   </si>
 </sst>
 </file>
@@ -1259,7 +1409,7 @@
         <v>3</v>
       </c>
       <c r="M5" s="27" t="n">
-        <v>14.25</v>
+        <v>14.5</v>
       </c>
       <c r="N5" s="27" t="s">
         <v>4</v>
@@ -1272,7 +1422,7 @@
         <v>5</v>
       </c>
       <c r="T5" s="27" t="n">
-        <v>6.75</v>
+        <v>6.5</v>
       </c>
       <c r="U5" s="27" t="s">
         <v>4</v>
@@ -1415,7 +1565,7 @@
         <v>10</v>
       </c>
       <c r="M9" s="27" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N9" s="27"/>
       <c r="O9" s="27"/>
@@ -1426,7 +1576,7 @@
         <v>11</v>
       </c>
       <c r="T9" s="27" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U9" s="27"/>
       <c r="V9" s="27"/>
@@ -1456,25 +1606,31 @@
         <v>12</v>
       </c>
       <c r="M10" s="27" t="n">
-        <v>0.089</v>
+        <f aca="false">VLOOKUP(O10,lists!$C$2:$D$49,2,0)</f>
+        <v>0.055</v>
       </c>
       <c r="N10" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="O10" s="27"/>
+      <c r="O10" s="27" t="s">
+        <v>13</v>
+      </c>
       <c r="P10" s="21"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="22"/>
       <c r="S10" s="27" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T10" s="27" t="n">
-        <v>0.05</v>
+        <f aca="false">VLOOKUP(V10,lists!$C$2:$D$49,2,0)</f>
+        <v>0.03125</v>
       </c>
       <c r="U10" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="V10" s="27"/>
+      <c r="V10" s="27" t="s">
+        <v>15</v>
+      </c>
       <c r="W10" s="26"/>
       <c r="X10" s="3"/>
       <c r="Y10" s="4"/>
@@ -1498,28 +1654,28 @@
       <c r="I11" s="16"/>
       <c r="K11" s="17"/>
       <c r="L11" s="29" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="M11" s="30" t="n">
         <f aca="false">PI()/4*M10^2*M9</f>
-        <v>0.0248845554090847</v>
+        <v>0.0142549766656637</v>
       </c>
       <c r="N11" s="29" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="O11" s="29"/>
       <c r="P11" s="21"/>
       <c r="Q11" s="3"/>
       <c r="R11" s="22"/>
       <c r="S11" s="29" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T11" s="30" t="n">
         <f aca="false">PI()/4*T10^2*T9</f>
-        <v>0.00785398163397448</v>
+        <v>0.00460194236365692</v>
       </c>
       <c r="U11" s="29" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="V11" s="29"/>
       <c r="W11" s="26"/>
@@ -1578,7 +1734,7 @@
       <c r="I13" s="16"/>
       <c r="K13" s="17"/>
       <c r="L13" s="18" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="M13" s="19"/>
       <c r="N13" s="19"/>
@@ -1587,7 +1743,7 @@
       <c r="Q13" s="3"/>
       <c r="R13" s="22"/>
       <c r="S13" s="23" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="T13" s="24"/>
       <c r="U13" s="24"/>
@@ -1615,7 +1771,7 @@
       <c r="I14" s="16"/>
       <c r="K14" s="17"/>
       <c r="L14" s="27" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M14" s="27" t="n">
         <v>12</v>
@@ -1628,7 +1784,7 @@
       <c r="Q14" s="3"/>
       <c r="R14" s="22"/>
       <c r="S14" s="27" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="T14" s="27" t="n">
         <v>36</v>
@@ -1660,7 +1816,7 @@
       <c r="I15" s="16"/>
       <c r="K15" s="17"/>
       <c r="L15" s="27" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="M15" s="27" t="n">
         <v>0.3125</v>
@@ -1673,7 +1829,7 @@
       <c r="Q15" s="3"/>
       <c r="R15" s="22"/>
       <c r="S15" s="27" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="T15" s="27" t="n">
         <v>0.225</v>
@@ -1705,7 +1861,7 @@
       <c r="I16" s="16"/>
       <c r="K16" s="17"/>
       <c r="L16" s="27" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="M16" s="31" t="n">
         <v>3.94E-006</v>
@@ -1718,7 +1874,7 @@
       <c r="Q16" s="3"/>
       <c r="R16" s="22"/>
       <c r="S16" s="27" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="T16" s="31" t="n">
         <v>3.94E-006</v>
@@ -1750,7 +1906,7 @@
       <c r="I17" s="16"/>
       <c r="K17" s="17"/>
       <c r="L17" s="27" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M17" s="27" t="n">
         <v>0.5</v>
@@ -1761,7 +1917,7 @@
       <c r="Q17" s="3"/>
       <c r="R17" s="22"/>
       <c r="S17" s="27" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="T17" s="27" t="n">
         <v>0.5</v>
@@ -1791,7 +1947,7 @@
       <c r="I18" s="36"/>
       <c r="K18" s="17"/>
       <c r="L18" s="27" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M18" s="27" t="n">
         <v>1.6</v>
@@ -1802,7 +1958,7 @@
       <c r="Q18" s="3"/>
       <c r="R18" s="22"/>
       <c r="S18" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="T18" s="27" t="n">
         <v>1.6</v>
@@ -1823,11 +1979,11 @@
     </row>
     <row r="19" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="37" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K19" s="17"/>
       <c r="L19" s="27" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="M19" s="27" t="n">
         <v>0</v>
@@ -1838,7 +1994,7 @@
       <c r="Q19" s="3"/>
       <c r="R19" s="22"/>
       <c r="S19" s="27" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T19" s="27" t="n">
         <v>2</v>
@@ -1868,7 +2024,7 @@
       <c r="I20" s="40"/>
       <c r="K20" s="17"/>
       <c r="L20" s="27" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M20" s="27" t="n">
         <v>0.8</v>
@@ -1879,7 +2035,7 @@
       <c r="Q20" s="3"/>
       <c r="R20" s="22"/>
       <c r="S20" s="27" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="T20" s="27" t="n">
         <v>0.8</v>
@@ -1901,7 +2057,7 @@
     <row r="21" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="41"/>
       <c r="C21" s="42" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D21" s="43"/>
       <c r="E21" s="43"/>
@@ -1917,13 +2073,13 @@
       <c r="P21" s="47"/>
       <c r="R21" s="22"/>
       <c r="S21" s="27" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="T21" s="27" t="n">
         <v>15</v>
       </c>
       <c r="U21" s="27" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="V21" s="27"/>
       <c r="W21" s="26"/>
@@ -1941,22 +2097,22 @@
     <row r="22" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="41"/>
       <c r="C22" s="27" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D22" s="48" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E22" s="49" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F22" s="48" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G22" s="27" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H22" s="27" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I22" s="44"/>
       <c r="R22" s="50"/>
@@ -1979,7 +2135,7 @@
     <row r="23" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="41"/>
       <c r="C23" s="27" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D23" s="53" t="n">
         <v>1</v>
@@ -1991,7 +2147,7 @@
         <v>0.1</v>
       </c>
       <c r="G23" s="54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H23" s="27" t="n">
         <f aca="false">(E23-D23)/F23 + 1</f>
@@ -2012,7 +2168,7 @@
     <row r="24" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="41"/>
       <c r="C24" s="27" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D24" s="53" t="n">
         <v>0.6</v>
@@ -2024,7 +2180,7 @@
         <v>0.1</v>
       </c>
       <c r="G24" s="54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H24" s="27" t="n">
         <f aca="false">(E24-D24)/F24 + 1</f>
@@ -2033,7 +2189,7 @@
       <c r="I24" s="44"/>
       <c r="K24" s="41"/>
       <c r="L24" s="55" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="M24" s="56"/>
       <c r="N24" s="56"/>
@@ -2057,7 +2213,7 @@
       <c r="I25" s="44"/>
       <c r="K25" s="41"/>
       <c r="L25" s="27" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="M25" s="27" t="n">
         <v>3</v>
@@ -2076,14 +2232,14 @@
     <row r="26" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="41"/>
       <c r="C26" s="55" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D26" s="59" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E26" s="59"/>
       <c r="F26" s="59" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G26" s="59"/>
       <c r="H26" s="60" t="s">
@@ -2092,7 +2248,7 @@
       <c r="I26" s="44"/>
       <c r="K26" s="41"/>
       <c r="L26" s="27" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M26" s="27" t="n">
         <v>0.065</v>
@@ -2111,13 +2267,13 @@
     <row r="27" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="41"/>
       <c r="C27" s="27" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D27" s="27" t="n">
         <v>0.01</v>
       </c>
       <c r="E27" s="27" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F27" s="27"/>
       <c r="G27" s="27"/>
@@ -2125,7 +2281,7 @@
       <c r="I27" s="44"/>
       <c r="K27" s="41"/>
       <c r="L27" s="27" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="M27" s="27" t="n">
         <v>1.5</v>
@@ -2144,13 +2300,13 @@
     <row r="28" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="41"/>
       <c r="C28" s="27" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D28" s="27" t="n">
         <v>30</v>
       </c>
       <c r="E28" s="27" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F28" s="27"/>
       <c r="G28" s="27"/>
@@ -2158,7 +2314,7 @@
       <c r="I28" s="44"/>
       <c r="K28" s="41"/>
       <c r="L28" s="27" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M28" s="27" t="n">
         <v>3</v>
@@ -2177,28 +2333,28 @@
     <row r="29" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="41"/>
       <c r="C29" s="27" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D29" s="27" t="n">
         <v>50</v>
       </c>
       <c r="E29" s="27" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F29" s="62" t="n">
         <f aca="false">(D29-32)/1.8</f>
         <v>10</v>
       </c>
       <c r="G29" s="27" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H29" s="27" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I29" s="44"/>
       <c r="K29" s="41"/>
       <c r="L29" s="27" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M29" s="27" t="n">
         <v>0.04</v>
@@ -2217,28 +2373,28 @@
     <row r="30" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="41"/>
       <c r="C30" s="27" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D30" s="27" t="n">
         <v>13.5</v>
       </c>
       <c r="E30" s="27" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F30" s="27" t="n">
         <f aca="false">D30*6895</f>
         <v>93082.5</v>
       </c>
       <c r="G30" s="27" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H30" s="27" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I30" s="44"/>
       <c r="K30" s="41"/>
       <c r="L30" s="27" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M30" s="63" t="n">
         <f aca="false">2*M27 + M5+T5</f>
@@ -2266,15 +2422,15 @@
       <c r="I31" s="44"/>
       <c r="K31" s="41"/>
       <c r="L31" s="27" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="M31" s="64" t="n">
         <f aca="false">M5/T5</f>
-        <v>2.11111111111111</v>
+        <v>2.23076923076923</v>
       </c>
       <c r="N31" s="27"/>
       <c r="O31" s="27" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="P31" s="44"/>
       <c r="Q31" s="61"/>
@@ -2286,7 +2442,7 @@
     <row r="32" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="41"/>
       <c r="C32" s="42" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D32" s="43"/>
       <c r="E32" s="43"/>
@@ -2296,17 +2452,17 @@
       <c r="I32" s="44"/>
       <c r="K32" s="41"/>
       <c r="L32" s="27" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="M32" s="63" t="n">
         <f aca="false">M27+M5-M28</f>
-        <v>12.75</v>
+        <v>13</v>
       </c>
       <c r="N32" s="27" t="s">
         <v>4</v>
       </c>
       <c r="O32" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="P32" s="44"/>
       <c r="Q32" s="3"/>
@@ -2318,10 +2474,10 @@
     <row r="33" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="41"/>
       <c r="C33" s="27" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D33" s="65" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E33" s="65"/>
       <c r="F33" s="66"/>
@@ -2336,7 +2492,7 @@
       <c r="P33" s="44"/>
       <c r="Q33" s="3"/>
       <c r="T33" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="Y33" s="2"/>
       <c r="AF33" s="2"/>
@@ -2345,7 +2501,7 @@
     <row r="34" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="41"/>
       <c r="C34" s="27" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D34" s="27"/>
       <c r="E34" s="27"/>
@@ -2353,13 +2509,13 @@
         <v>786</v>
       </c>
       <c r="G34" s="27" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H34" s="27"/>
       <c r="I34" s="44"/>
       <c r="K34" s="41"/>
       <c r="L34" s="55" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="M34" s="56"/>
       <c r="N34" s="56"/>
@@ -2373,7 +2529,7 @@
     <row r="35" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="41"/>
       <c r="C35" s="27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D35" s="27"/>
       <c r="E35" s="27"/>
@@ -2381,13 +2537,13 @@
         <v>2.5</v>
       </c>
       <c r="G35" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H35" s="27"/>
       <c r="I35" s="44"/>
       <c r="K35" s="67"/>
       <c r="L35" s="27" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M35" s="27" t="n">
         <v>1.5</v>
@@ -2405,7 +2561,7 @@
     <row r="36" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="41"/>
       <c r="C36" s="27" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D36" s="27"/>
       <c r="E36" s="27"/>
@@ -2413,15 +2569,15 @@
         <v>0.07</v>
       </c>
       <c r="G36" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H36" s="27" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I36" s="44"/>
       <c r="K36" s="67"/>
       <c r="L36" s="27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="M36" s="27" t="n">
         <v>0.25</v>
@@ -2446,7 +2602,7 @@
       <c r="I37" s="44"/>
       <c r="K37" s="67"/>
       <c r="L37" s="27" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M37" s="27" t="n">
         <v>4</v>
@@ -2463,7 +2619,7 @@
     <row r="38" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="41"/>
       <c r="C38" s="55" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D38" s="56"/>
       <c r="E38" s="56"/>
@@ -2481,7 +2637,7 @@
     <row r="39" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="41"/>
       <c r="C39" s="27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D39" s="27" t="n">
         <v>0.65</v>
@@ -2493,7 +2649,7 @@
       <c r="I39" s="44"/>
       <c r="K39" s="67"/>
       <c r="L39" s="55" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="M39" s="56"/>
       <c r="N39" s="56"/>
@@ -2503,7 +2659,7 @@
     <row r="40" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="41"/>
       <c r="C40" s="27" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D40" s="27" t="n">
         <v>0.95</v>
@@ -2515,7 +2671,7 @@
       <c r="I40" s="44"/>
       <c r="K40" s="41"/>
       <c r="L40" s="27" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M40" s="27" t="n">
         <v>0.75</v>
@@ -2529,7 +2685,7 @@
     <row r="41" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="41"/>
       <c r="C41" s="27" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D41" s="27" t="n">
         <v>0.7</v>
@@ -2541,10 +2697,10 @@
       <c r="I41" s="44"/>
       <c r="K41" s="41"/>
       <c r="L41" s="27" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M41" s="27" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="N41" s="27" t="s">
         <v>4</v>
@@ -2555,13 +2711,13 @@
     <row r="42" customFormat="false" ht="15.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="41"/>
       <c r="C42" s="27" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D42" s="27" t="n">
         <v>0.25</v>
       </c>
       <c r="E42" s="27" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F42" s="27"/>
       <c r="G42" s="27"/>
@@ -2569,13 +2725,13 @@
       <c r="I42" s="44"/>
       <c r="K42" s="41"/>
       <c r="L42" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="M42" s="27" t="n">
         <v>15</v>
       </c>
       <c r="N42" s="27" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="O42" s="27"/>
       <c r="P42" s="44"/>
@@ -2604,7 +2760,7 @@
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="F33:H33"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D33" type="list">
       <formula1>"Isopropanol,Ethanol,E98,E85"</formula1>
       <formula2>0</formula2>
@@ -2625,6 +2781,10 @@
       <formula1>lists!$A$2:$A$43</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation allowBlank="false" error="Pick a drill size from the list." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="O10 V10" type="list">
+      <formula1>lists!$C$2:$C$49</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -2641,233 +2801,534 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A200"/>
+  <dimension ref="A1:D200"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="45.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="41.49"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0.0135</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0.0145</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0.015625</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0.016</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0.018</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0.02</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0.021</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>0.0225</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0.024</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>0.025</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>0.026</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="C13" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>0.028</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="C14" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>0.0292</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="C15" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>0.031</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="C16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>0.03125</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>0.032</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>0.033</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>0.035</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>0.036</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>0.037</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>0.038</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>0.039</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>0.04</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>0.041</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>0.042</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>0.043</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>0.0465</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>0.046875</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>0.052</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>0.055</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="C32" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>0.0595</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="C33" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>0.0625</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="C34" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>0.0635</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>0.067</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>0.07</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>0.073</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>0.076</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>0.078125</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>0.0785</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>0.081</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>0.082</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>37</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>0.086</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C44" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>0.089</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C45" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D45" s="1" t="n">
+        <v>0.0935</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C46" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D46" s="1" t="n">
+        <v>0.09375</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C47" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D47" s="1" t="n">
+        <v>0.096</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C48" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D48" s="1" t="n">
+        <v>0.098</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C49" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D49" s="1" t="n">
+        <v>0.0995</v>
+      </c>
+    </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>